<commit_message>
Remove quoted notice passages from the public check files; the notice texts are kept for research only
</commit_message>
<xml_diff>
--- a/checks/11-check-sheet.filled.xlsx
+++ b/checks/11-check-sheet.filled.xlsx
@@ -644,7 +644,7 @@
       </c>
       <c r="G1" s="3" t="inlineStr">
         <is>
-          <t>evidence quote from the notice</t>
+          <t>evidence quote from the notice (removed in the public copy)</t>
         </is>
       </c>
       <c r="H1" s="3" t="inlineStr">
@@ -704,7 +704,7 @@
       </c>
       <c r="G2" s="2" t="inlineStr">
         <is>
-          <t>“The personal data collected may include: – Your name – Your billing / postal address – Your telephone number(s) – Your email address – Your photo – Records of your correspondence with us – Device ID”</t>
+          <t>[removed: notice text is kept for research only]</t>
         </is>
       </c>
       <c r="H2" s="2" t="inlineStr">
@@ -752,7 +752,7 @@
       </c>
       <c r="G3" s="2" t="inlineStr">
         <is>
-          <t>“In-order to facilitate our services and correspondence purposes we need to gather your own information. We guarantee that the data we gather and use is fitting for this reason. We are an organization which esteems its clients’ information security and protection privileges and we have no interest in gathering any information beyond what we need to make our service(s) work for you. We generally process your personal information for specific purposes with the nature of the information gathered relying upon your collaboration with us. We are focused on transparency in this regard”</t>
+          <t>[removed: notice text is kept for research only]</t>
         </is>
       </c>
       <c r="H3" s="2" t="inlineStr">
@@ -800,7 +800,7 @@
       </c>
       <c r="G4" s="2" t="inlineStr">
         <is>
-          <t>Closest text found (not necessarily enough for 'met'): “If you disagree with any changes to this Privacy Policy, you may choose to stop using the [NAME] Web Applications.”</t>
+          <t>[removed: notice text is kept for research only]</t>
         </is>
       </c>
       <c r="H4" s="2" t="inlineStr">
@@ -848,7 +848,7 @@
       </c>
       <c r="G5" s="2" t="inlineStr">
         <is>
-          <t>Closest text found (not necessarily enough for 'met'): “It’s significant that you read the full policy to know what data we hold, how we might utilize it, and what your privileges are – yet on the off chance that you don’t have the opportunity to peruse it all presently, here’s a speedy outline:”</t>
+          <t>[removed: notice text is kept for research only]</t>
         </is>
       </c>
       <c r="H5" s="2" t="inlineStr">
@@ -869,7 +869,7 @@
       </c>
       <c r="L5" s="5" t="inlineStr">
         <is>
-          <t>Lines 82-84: generic contact for inquiries (and line 91 refers to 'your privileges'); a 'contact us' means with no rights named = P under the rule.</t>
+          <t>Lines 82-84: generic contact for inquiries (and line 91 refers to [quote removed]); a [quote removed] means with no rights named = P under the rule.</t>
         </is>
       </c>
     </row>
@@ -904,7 +904,7 @@
       </c>
       <c r="G6" s="2" t="inlineStr">
         <is>
-          <t>no matching text found</t>
+          <t>[removed: notice text is kept for research only]</t>
         </is>
       </c>
       <c r="H6" s="2" t="inlineStr"/>
@@ -948,7 +948,7 @@
       </c>
       <c r="G7" s="2" t="inlineStr">
         <is>
-          <t>(whole notice) The notice text is in English.</t>
+          <t>[removed: notice text is kept for research only]</t>
         </is>
       </c>
       <c r="H7" s="2" t="inlineStr">
@@ -996,7 +996,7 @@
       </c>
       <c r="G8" s="2" t="inlineStr">
         <is>
-          <t>“Welcome to [NAME]! By utilizing our services (Web based, API based or other services or applications) you are consenting to our Terms of Service characterized in this document and the Cookie Policy incorporated by reference. Kindly read the Terms of Service cautiously prior to utilizing our services. Likewise, please read all policies and guidelines incorporated in our web application such as Privacy Policy and Cookie Policy, and contact [EMAIL] on the off chance that you have any inquiries.”</t>
+          <t>[removed: notice text is kept for research only]</t>
         </is>
       </c>
       <c r="H8" s="2" t="inlineStr">
@@ -1044,7 +1044,7 @@
       </c>
       <c r="G9" s="2" t="inlineStr">
         <is>
-          <t>no matching text found</t>
+          <t>[removed: notice text is kept for research only]</t>
         </is>
       </c>
       <c r="H9" s="2" t="inlineStr"/>
@@ -1088,7 +1088,7 @@
       </c>
       <c r="G10" s="2" t="inlineStr">
         <is>
-          <t>no matching text found</t>
+          <t>[removed: notice text is kept for research only]</t>
         </is>
       </c>
       <c r="H10" s="2" t="inlineStr"/>
@@ -1132,7 +1132,7 @@
       </c>
       <c r="G11" s="2" t="inlineStr">
         <is>
-          <t>“By signing up for an account you agree to these Terms of Service, and any additional terms specified by services (APIs, etc.) or applications that you elect to use. You also agree to our privacy policy, incorporated herein by reference. These Terms of Service, together with the Privacy Policy, Cookie Policy and any other terms contained herein or incorporated herein by reference, are jointly referred to as the “Terms of Service”. These Terms of Service apply to all services and users.”</t>
+          <t>[removed: notice text is kept for research only]</t>
         </is>
       </c>
       <c r="H11" s="2" t="inlineStr">
@@ -1180,7 +1180,7 @@
       </c>
       <c r="G12" s="2" t="inlineStr">
         <is>
-          <t>Closest text found (not necessarily enough for 'met'): “We gather data about each and every individual who accesses the [NAME]. This could be Faculty, Students, Employees, Parents and individuals who partake in our events, trustees or venture candidates for financing organizations.”</t>
+          <t>[removed: notice text is kept for research only]</t>
         </is>
       </c>
       <c r="H12" s="2" t="inlineStr">
@@ -1228,7 +1228,7 @@
       </c>
       <c r="G13" s="2" t="inlineStr">
         <is>
-          <t>no matching text found</t>
+          <t>[removed: notice text is kept for research only]</t>
         </is>
       </c>
       <c r="H13" s="2" t="inlineStr"/>
@@ -1272,7 +1272,7 @@
       </c>
       <c r="G14" s="2" t="inlineStr">
         <is>
-          <t>no matching text found</t>
+          <t>[removed: notice text is kept for research only]</t>
         </is>
       </c>
       <c r="H14" s="2" t="inlineStr"/>
@@ -1316,7 +1316,7 @@
       </c>
       <c r="G15" s="2" t="inlineStr">
         <is>
-          <t>no matching text found</t>
+          <t>[removed: notice text is kept for research only]</t>
         </is>
       </c>
       <c r="H15" s="2" t="inlineStr"/>
@@ -1360,7 +1360,7 @@
       </c>
       <c r="G16" s="2" t="inlineStr">
         <is>
-          <t>Closest text found (not necessarily enough for 'met'): “Our services use Cookies and the security measure is trailed by Cookie Policy incorporated by reference herein The third-party applications might gather data used to identify you.”</t>
+          <t>[removed: notice text is kept for research only]</t>
         </is>
       </c>
       <c r="H16" s="2" t="inlineStr">
@@ -1408,7 +1408,7 @@
       </c>
       <c r="G17" s="2" t="inlineStr">
         <is>
-          <t>“If you contact us directly, we may receive additional information about you such as your name, email address, phone number, the contents of the message and/or attachments you may send us, and any other information you may choose to provide. When you register for an Account, we may ask for your contact information, including items such as name, company name, address, email address, and telephone number.”</t>
+          <t>[removed: notice text is kept for research only]</t>
         </is>
       </c>
       <c r="H17" s="2" t="inlineStr">
@@ -1456,7 +1456,7 @@
       </c>
       <c r="G18" s="2" t="inlineStr">
         <is>
-          <t>“We use the information we collect in various ways, including to: Provide, operate, and maintain our website Improve, personalize, and expand our website Understand and analyze how you use our website Develop new products, services, features, and functionality Communicate with you, either directly or through one of our partners, including for customer service, to provide you with updates and other information relating to the website, and for marketing and promotional purposes Send you emails Find and prevent fraud”</t>
+          <t>[removed: notice text is kept for research only]</t>
         </is>
       </c>
       <c r="H18" s="2" t="inlineStr">
@@ -1504,7 +1504,7 @@
       </c>
       <c r="G19" s="2" t="inlineStr">
         <is>
-          <t>Closest text found (not necessarily enough for 'met'): “and other sites on the internet. However, visitors may choose to decline the use of DART cookies by visiting the Google ad and content network Privacy Policy at the following URL –”</t>
+          <t>[removed: notice text is kept for research only]</t>
         </is>
       </c>
       <c r="H19" s="2" t="inlineStr">
@@ -1552,7 +1552,7 @@
       </c>
       <c r="G20" s="2" t="inlineStr">
         <is>
-          <t>“The right to rectification – You have the right to request that we correct any information you believe is inaccurate. You also have the right to request that we complete the information you believe is incomplete. If you make a request, we have one month to respond to you. If you would like to exercise any of these rights, please contact us at [EMAIL].”</t>
+          <t>[removed: notice text is kept for research only]</t>
         </is>
       </c>
       <c r="H20" s="2" t="inlineStr">
@@ -1600,7 +1600,7 @@
       </c>
       <c r="G21" s="2" t="inlineStr">
         <is>
-          <t>no matching text found</t>
+          <t>[removed: notice text is kept for research only]</t>
         </is>
       </c>
       <c r="H21" s="2" t="inlineStr"/>
@@ -1644,7 +1644,7 @@
       </c>
       <c r="G22" s="2" t="inlineStr">
         <is>
-          <t>(whole notice) The notice text is in English.</t>
+          <t>[removed: notice text is kept for research only]</t>
         </is>
       </c>
       <c r="H22" s="2" t="inlineStr">
@@ -1692,7 +1692,7 @@
       </c>
       <c r="G23" s="2" t="inlineStr">
         <is>
-          <t>“If you have additional questions or require more information about our Privacy Policy, do not hesitate to contact us through email at [EMAIL]”</t>
+          <t>[removed: notice text is kept for research only]</t>
         </is>
       </c>
       <c r="H23" s="2" t="inlineStr">
@@ -1740,7 +1740,7 @@
       </c>
       <c r="G24" s="2" t="inlineStr">
         <is>
-          <t>Closest text found (not necessarily enough for 'met'): “If you make a request, we have one month to respond to you. If you would like to exercise any of these rights, please contact us at [EMAIL].”</t>
+          <t>[removed: notice text is kept for research only]</t>
         </is>
       </c>
       <c r="H24" s="2" t="inlineStr">
@@ -1788,7 +1788,7 @@
       </c>
       <c r="G25" s="2" t="inlineStr">
         <is>
-          <t>Closest text found (not necessarily enough for 'met'): “If you make a request, we have one month to respond to you. If you would like to exercise any of these rights, please contact us at [EMAIL].”</t>
+          <t>[removed: notice text is kept for research only]</t>
         </is>
       </c>
       <c r="H25" s="2" t="inlineStr">
@@ -1809,7 +1809,7 @@
       </c>
       <c r="L25" s="5" t="inlineStr">
         <is>
-          <t>Lines 49 and 58: 'we have one month to respond' to rights requests; rule v1.1 counts rights requests.</t>
+          <t>Lines 49 and 58: [quote removed] to rights requests; rule v1.1 counts rights requests.</t>
         </is>
       </c>
     </row>
@@ -1844,7 +1844,7 @@
       </c>
       <c r="G26" s="2" t="inlineStr">
         <is>
-          <t>“, one of our main priorities is the privacy of our visitors. This Privacy Policy document contains types of information that is collected and recorded by [NAME] and how we use it.”</t>
+          <t>[removed: notice text is kept for research only]</t>
         </is>
       </c>
       <c r="H26" s="2" t="inlineStr">
@@ -1892,7 +1892,7 @@
       </c>
       <c r="G27" s="2" t="inlineStr">
         <is>
-          <t>“Children’s Information Another part of our priority is adding protection for children while using the internet. We encourage parents and guardians to observe, participate in, and/or monitor and guide their online activity.”</t>
+          <t>[removed: notice text is kept for research only]</t>
         </is>
       </c>
       <c r="H27" s="2" t="inlineStr">
@@ -1940,7 +1940,7 @@
       </c>
       <c r="G28" s="2" t="inlineStr">
         <is>
-          <t>“[NAME] does not knowingly collect any Personal Identifiable Information from children under the age of 13. If you think that your child provided this kind of information on our website, we strongly encourage you to contact us immediately and we will do our best efforts to promptly remove such information from our records.”</t>
+          <t>[removed: notice text is kept for research only]</t>
         </is>
       </c>
       <c r="H28" s="2" t="inlineStr">
@@ -1988,7 +1988,7 @@
       </c>
       <c r="G29" s="2" t="inlineStr">
         <is>
-          <t>Closest text found (not necessarily enough for 'met'): “Another part of our priority is adding protection for children while using the internet. We encourage parents and guardians to observe, participate in, and/or monitor and guide their online activity. [NAME] does not knowingly collect any Personal Identifiable Information from children under the age of 13. If you think that your child provided this kind of information on our website, we strongly encourage you to contact us immediately and we will do our best efforts to promptly remove such information from our records.”</t>
+          <t>[removed: notice text is kept for research only]</t>
         </is>
       </c>
       <c r="H29" s="2" t="inlineStr">
@@ -2009,7 +2009,7 @@
       </c>
       <c r="L29" s="5" t="inlineStr">
         <is>
-          <t>Line 61: parents told to contact the school if their child provided data, so it can be removed = parents 'may contact' (P).</t>
+          <t>Line 61: parents told to contact the school if their child provided data, so it can be removed = parents [quote removed] (P).</t>
         </is>
       </c>
     </row>
@@ -2044,7 +2044,7 @@
       </c>
       <c r="G30" s="2" t="inlineStr">
         <is>
-          <t>no matching text found</t>
+          <t>[removed: notice text is kept for research only]</t>
         </is>
       </c>
       <c r="H30" s="2" t="inlineStr"/>
@@ -2088,7 +2088,7 @@
       </c>
       <c r="G31" s="2" t="inlineStr">
         <is>
-          <t>Closest text found (not necessarily enough for 'met'): “Google is one of the third-party vendors on our site. It also uses cookies, known as DART cookies, to serve ads to our site visitors based upon their visit to [URL] and other sites on the internet. However, visitors may choose to decline the use of DART cookies by visiting the Google ad and content network Privacy Policy at the following URL – Third-party ad servers or ad networks use technologies like cookies, JavaScript, or Web Beacons that are used in their respective advertisements and links that appear on [NAME], which are sent directly to users’ browsers. They automatically receive your IP address when this occurs. These technologies are used to measure the effectiveness of their advertising campaigns and/or to personalize the advertising content that you see on websites that you visit.”</t>
+          <t>[removed: notice text is kept for research only]</t>
         </is>
       </c>
       <c r="H31" s="2" t="inlineStr">
@@ -2136,7 +2136,7 @@
       </c>
       <c r="G32" s="2" t="inlineStr">
         <is>
-          <t>“When you use the Website [URL] (A unit of [NAME] educational Society), we collect and store your personal information which is provided by you from time to time. Our primary goal in doing so is to We may use your personal information, including date of birth, to verify identity, assist with identification of users, and to determine appropriate services. We may collect information such as occupation, language, zip code, area code, , referrer URL, location, and the time zone where [NAME] school product and/or service is used so that we can better understand customer”</t>
+          <t>[removed: notice text is kept for research only]</t>
         </is>
       </c>
       <c r="H32" s="2" t="inlineStr">
@@ -2192,7 +2192,7 @@
       </c>
       <c r="G33" s="2" t="inlineStr">
         <is>
-          <t>“The personal information we collect allows us to keep you posted on [NAME] school’s latest product announcements, offers, and upcoming events. We also use personal information to help us create, develop, operate, deliver, and improve our products, services, content and advertising, and for loss prevention and anti-fraud purposes.”</t>
+          <t>[removed: notice text is kept for research only]</t>
         </is>
       </c>
       <c r="H33" s="2" t="inlineStr">
@@ -2240,7 +2240,7 @@
       </c>
       <c r="G34" s="2" t="inlineStr">
         <is>
-          <t>Closest text found (not necessarily enough for 'met'): “From time to time, we may use your personal information to send important notices, such as communications about purchases and changes to our terms, conditions, and policies. Please note as this information is important to your interaction with [NAME] school, you may not opt out of receiving these communications.”</t>
+          <t>[removed: notice text is kept for research only]</t>
         </is>
       </c>
       <c r="H34" s="2" t="inlineStr">
@@ -2288,7 +2288,7 @@
       </c>
       <c r="G35" s="2" t="inlineStr">
         <is>
-          <t>“ACCESS TO PERSONAL INFORMATION You can help ensure that your contact information and preferences are accurate, complete, and up to date by logging in to your account. For other personal information we hold, we will provide you with access for any purpose including to request that we correct the data if it is inaccurate or delete the data if [NAME] school is not required to retain it by law or for legitimate business purposes. We may decline to process requests that”</t>
+          <t>[removed: notice text is kept for research only]</t>
         </is>
       </c>
       <c r="H35" s="2" t="inlineStr">
@@ -2305,7 +2305,7 @@
       <c r="K35" s="5" t="n"/>
       <c r="L35" s="5" t="inlineStr">
         <is>
-          <t>Rights to access, correct and delete are named (lines 106-108); the only means are account login for contact details (lines 105-106) and the general 'contact us' (lines 129-132). Unsure whether that is a means to request the rights (Y) or rights with no means (P).</t>
+          <t>Rights to access, correct and delete are named (lines 106-108); the only means are account login for contact details (lines 105-106) and the general [quote removed] (lines 129-132). Unsure whether that is a means to request the rights (Y) or rights with no means (P).</t>
         </is>
       </c>
     </row>
@@ -2340,7 +2340,7 @@
       </c>
       <c r="G36" s="2" t="inlineStr">
         <is>
-          <t>Closest text found (not necessarily enough for 'met'): “All such communications are examined and replies issued where appropriate as soon as possible. If you are unsatisfied with the reply received, you may refer your complaint to the relevant regulator in your jurisdiction. If you ask us, we will endeavor to provide you with information about relevant complaint avenues which may be applicable to your circumstances.”</t>
+          <t>[removed: notice text is kept for research only]</t>
         </is>
       </c>
       <c r="H36" s="2" t="inlineStr">
@@ -2361,7 +2361,7 @@
       </c>
       <c r="L36" s="5" t="inlineStr">
         <is>
-          <t>Line 134: unsatisfied users may refer the complaint to 'the relevant regulator in your jurisdiction' = generic regulator (P).</t>
+          <t>Line 134: unsatisfied users may refer the complaint to [quote removed] = generic regulator (P).</t>
         </is>
       </c>
     </row>
@@ -2396,7 +2396,7 @@
       </c>
       <c r="G37" s="2" t="inlineStr">
         <is>
-          <t>(whole notice) The notice text is in English.</t>
+          <t>[removed: notice text is kept for research only]</t>
         </is>
       </c>
       <c r="H37" s="2" t="inlineStr">
@@ -2444,7 +2444,7 @@
       </c>
       <c r="G38" s="2" t="inlineStr">
         <is>
-          <t>“Grievance Redressal Redressal Mechanism: Any complaints, abuse or concerns with regards to content and or comment or breach of these terms shall be immediately informed to the designated Grievance Officer as mentioned below via in writing or through email signed with the electronic signature to Mr. [NAME] ("Grievance Officer"). Mr. [NAME] (Grievance Officer) [URL] [NAME] school, [NAME], New Delhi-110071 Email: [EMAIL]”</t>
+          <t>[removed: notice text is kept for research only]</t>
         </is>
       </c>
       <c r="H38" s="2" t="inlineStr">
@@ -2492,7 +2492,7 @@
       </c>
       <c r="G39" s="2" t="inlineStr">
         <is>
-          <t>“Grievance Redressal Redressal Mechanism: Any complaints, abuse or concerns with regards to content and or comment or breach of these terms shall be immediately informed to the designated Grievance Officer as mentioned below via in writing or through email signed with the electronic signature to Mr. [NAME] ("Grievance Officer").”</t>
+          <t>[removed: notice text is kept for research only]</t>
         </is>
       </c>
       <c r="H39" s="2" t="inlineStr">
@@ -2540,7 +2540,7 @@
       </c>
       <c r="G40" s="2" t="inlineStr">
         <is>
-          <t>Closest text found (not necessarily enough for 'met'): “All such communications are examined and replies issued where appropriate as soon as possible. If you are”</t>
+          <t>[removed: notice text is kept for research only]</t>
         </is>
       </c>
       <c r="H40" s="2" t="inlineStr">
@@ -2588,7 +2588,7 @@
       </c>
       <c r="G41" s="2" t="inlineStr">
         <is>
-          <t>“COLLECTION AND USE OF PERSONAL INFORMATION When you use the Website [URL] (A unit of [NAME] educational Society), we collect and store your personal information which is provided by you from time to time. Our primary goal in doing so is to provide you a safe, efficient, smooth and customized experience. This allows us to provide services and”</t>
+          <t>[removed: notice text is kept for research only]</t>
         </is>
       </c>
       <c r="H41" s="2" t="inlineStr">
@@ -2636,7 +2636,7 @@
       </c>
       <c r="G42" s="2" t="inlineStr">
         <is>
-          <t>no matching text found</t>
+          <t>[removed: notice text is kept for research only]</t>
         </is>
       </c>
       <c r="H42" s="2" t="inlineStr"/>
@@ -2680,7 +2680,7 @@
       </c>
       <c r="G43" s="2" t="inlineStr">
         <is>
-          <t>no matching text found</t>
+          <t>[removed: notice text is kept for research only]</t>
         </is>
       </c>
       <c r="H43" s="2" t="inlineStr"/>
@@ -2724,7 +2724,7 @@
       </c>
       <c r="G44" s="2" t="inlineStr">
         <is>
-          <t>no matching text found</t>
+          <t>[removed: notice text is kept for research only]</t>
         </is>
       </c>
       <c r="H44" s="2" t="inlineStr"/>
@@ -2768,7 +2768,7 @@
       </c>
       <c r="G45" s="2" t="inlineStr">
         <is>
-          <t>no matching text found</t>
+          <t>[removed: notice text is kept for research only]</t>
         </is>
       </c>
       <c r="H45" s="2" t="inlineStr"/>
@@ -2812,7 +2812,7 @@
       </c>
       <c r="G46" s="2" t="inlineStr">
         <is>
-          <t>Closest text found (not necessarily enough for 'met'): “We may automatically track certain information about you based upon your behaviour on our Website. We use this information to do internal research on our users’ demographics, interests, and behaviour to better understand, protect and serve our users. This information is compiled and analysed on an aggregated basis. This”</t>
+          <t>[removed: notice text is kept for research only]</t>
         </is>
       </c>
       <c r="H46" s="2" t="inlineStr">
@@ -2860,7 +2860,7 @@
       </c>
       <c r="G47" s="2" t="inlineStr">
         <is>
-          <t>“While using our Service, we may ask you to provide us with certain personally identifiable information that can be used to contact or identify you (“Personal Data”). Personally identifiable information may include, but is not limited to: • Email address • First name and last name • Phone number • Address, State, Province, ZIP/Postal code, City”</t>
+          <t>[removed: notice text is kept for research only]</t>
         </is>
       </c>
       <c r="H47" s="2" t="inlineStr">
@@ -2908,7 +2908,7 @@
       </c>
       <c r="G48" s="2" t="inlineStr">
         <is>
-          <t>“[NAME] uses the collected data for various purposes: • To provide and maintain the Service • To notify you about changes to our Service • To allow you to participate in interactive features of our Service when you choose to do so • To provide customer care and support • To provide analysis or valuable information so that we can improve the Service • To monitor the usage of the Service • To detect, prevent and address technical issues”</t>
+          <t>[removed: notice text is kept for research only]</t>
         </is>
       </c>
       <c r="H48" s="2" t="inlineStr">
@@ -2956,7 +2956,7 @@
       </c>
       <c r="G49" s="2" t="inlineStr">
         <is>
-          <t>Closest text found (not necessarily enough for 'met'): “You can opt-out of having made your activity on the Service available to Google Analytics by installing the Google Analytics opt-out browser add-on. The add-on prevents the Google Analytics JavaScript (ga.js, analytics.js, and dc.js) from sharing information with Google Analytics about visits activity.”</t>
+          <t>[removed: notice text is kept for research only]</t>
         </is>
       </c>
       <c r="H49" s="2" t="inlineStr">
@@ -3004,7 +3004,7 @@
       </c>
       <c r="G50" s="2" t="inlineStr">
         <is>
-          <t>Closest text found (not necessarily enough for 'met'): “This page informs you of our policies regarding the collection, use, and disclosure of personal data when you use our Service and the choices you have associated with that data. Our Privacy Policy for [NAME] is based on the companies’ internal business norms.”</t>
+          <t>[removed: notice text is kept for research only]</t>
         </is>
       </c>
       <c r="H50" s="2" t="inlineStr">
@@ -3060,7 +3060,7 @@
       </c>
       <c r="G51" s="2" t="inlineStr">
         <is>
-          <t>no matching text found</t>
+          <t>[removed: notice text is kept for research only]</t>
         </is>
       </c>
       <c r="H51" s="2" t="inlineStr"/>
@@ -3104,7 +3104,7 @@
       </c>
       <c r="G52" s="2" t="inlineStr">
         <is>
-          <t>(whole notice) The notice text is in English.</t>
+          <t>[removed: notice text is kept for research only]</t>
         </is>
       </c>
       <c r="H52" s="2" t="inlineStr">
@@ -3152,7 +3152,7 @@
       </c>
       <c r="G53" s="2" t="inlineStr">
         <is>
-          <t>“Should you have any questions about this Privacy Policy, please contact us: • By email: [EMAIL]”</t>
+          <t>[removed: notice text is kept for research only]</t>
         </is>
       </c>
       <c r="H53" s="2" t="inlineStr">
@@ -3200,7 +3200,7 @@
       </c>
       <c r="G54" s="2" t="inlineStr">
         <is>
-          <t>no matching text found</t>
+          <t>[removed: notice text is kept for research only]</t>
         </is>
       </c>
       <c r="H54" s="2" t="inlineStr"/>
@@ -3244,7 +3244,7 @@
       </c>
       <c r="G55" s="2" t="inlineStr">
         <is>
-          <t>no matching text found</t>
+          <t>[removed: notice text is kept for research only]</t>
         </is>
       </c>
       <c r="H55" s="2" t="inlineStr"/>
@@ -3288,7 +3288,7 @@
       </c>
       <c r="G56" s="2" t="inlineStr">
         <is>
-          <t>“This page informs you of our policies regarding the collection, use, and disclosure of personal data when you use our Service and the choices you have associated with that data. Our Privacy Policy for [NAME] is based on the companies’ internal business norms.”</t>
+          <t>[removed: notice text is kept for research only]</t>
         </is>
       </c>
       <c r="H56" s="2" t="inlineStr">
@@ -3336,7 +3336,7 @@
       </c>
       <c r="G57" s="2" t="inlineStr">
         <is>
-          <t>“We do not knowingly collect personally identifiable information from anyone under the age of 18, unless otherwise approved by the Parent or Guardian. If you are a parent or guardian and you are aware that your children have provided us with Personal Data, please contact us. If we become aware that we have collected Personal Data from children without verification of parental consent, we take steps to remove that information from our servers.”</t>
+          <t>[removed: notice text is kept for research only]</t>
         </is>
       </c>
       <c r="H57" s="2" t="inlineStr">
@@ -3384,7 +3384,7 @@
       </c>
       <c r="G58" s="2" t="inlineStr">
         <is>
-          <t>“We do not knowingly collect personally identifiable information from anyone under the age of 18, unless otherwise approved by the Parent or Guardian. If you are a parent or guardian and you are aware that your children have provided us with Personal Data, please contact us. If we become aware that we have collected Personal Data from children without verification of parental consent, we take steps to remove that information from our servers.”</t>
+          <t>[removed: notice text is kept for research only]</t>
         </is>
       </c>
       <c r="H58" s="2" t="inlineStr">
@@ -3432,7 +3432,7 @@
       </c>
       <c r="G59" s="2" t="inlineStr">
         <is>
-          <t>“We do not knowingly collect personally identifiable information from anyone under the age of 18, unless otherwise approved by the Parent or Guardian. If you are a parent or guardian and you are aware that your children have provided us with Personal Data, please contact us. If we become aware that we have collected Personal Data from children without verification of parental consent, we take steps to remove that information from our servers.”</t>
+          <t>[removed: notice text is kept for research only]</t>
         </is>
       </c>
       <c r="H59" s="2" t="inlineStr">
@@ -3453,7 +3453,7 @@
       </c>
       <c r="L59" s="5" t="inlineStr">
         <is>
-          <t>Line 66: no collection from under-18s 'unless otherwise approved by the Parent or Guardian', data collected without verified parental consent is removed = consent required before processing.</t>
+          <t>Line 66: no collection from under-18s [quote removed], data collected without verified parental consent is removed = consent required before processing.</t>
         </is>
       </c>
     </row>
@@ -3488,7 +3488,7 @@
       </c>
       <c r="G60" s="2" t="inlineStr">
         <is>
-          <t>“We do not knowingly collect personally identifiable information from anyone under the age of 18, unless otherwise approved by the Parent or Guardian. If you are a parent or guardian and you are aware that your children have provided us with Personal Data, please contact us. If we become aware that we have collected Personal Data from children without verification of parental consent, we take steps to remove that information from our servers.”</t>
+          <t>[removed: notice text is kept for research only]</t>
         </is>
       </c>
       <c r="H60" s="2" t="inlineStr">
@@ -3536,7 +3536,7 @@
       </c>
       <c r="G61" s="2" t="inlineStr">
         <is>
-          <t>Closest text found (not necessarily enough for 'met'): “Google Analytics is a web analytics service offered by Google that tracks and reports website traffic. Google uses the data collected to track and monitor the use of our Service. This data is shared with other Google services. Google may use the collected data to contextualize and personalize the ads of its own advertising network.”</t>
+          <t>[removed: notice text is kept for research only]</t>
         </is>
       </c>
       <c r="H61" s="2" t="inlineStr">
@@ -3584,7 +3584,7 @@
       </c>
       <c r="G62" s="2" t="inlineStr">
         <is>
-          <t>“[NAME] may collect through some portions of the Website personal identifiable information, such as your name, address, telephone number, and email address (“Personal Information”). We may also collect anonymous demographic and usage pattern information which is not unique to you, such as your geographic area, age, gender, preferences, interests, favorites, log-in frequency, purchase history, and usage history. This demographic and usage pattern information is not considered Personal Information except when it is used in conjunction with other information that personally identifies you.”</t>
+          <t>[removed: notice text is kept for research only]</t>
         </is>
       </c>
       <c r="H62" s="2" t="inlineStr">
@@ -3632,7 +3632,7 @@
       </c>
       <c r="G63" s="2" t="inlineStr">
         <is>
-          <t>“We use your Personal Information to: (a) operate the Website and provide the services we offer; (b) deliver the services you request; (c) provide technical support; (d) verify any online payment, telephone payment, and pre-paid card transactions, which are solely processed through third-party service providers with their own privacy policies for which we are not responsible; (e) investigate alleged fraud, infringement, or other misconduct; (f) send you newsletters; and (g) inform you about other products, services, events, and promotions available from [NAME] or its affiliates. We may also use your Personal Information to contact you via surveys or other research regarding your opinion of any current and potential services.”</t>
+          <t>[removed: notice text is kept for research only]</t>
         </is>
       </c>
       <c r="H63" s="2" t="inlineStr">
@@ -3680,7 +3680,7 @@
       </c>
       <c r="G64" s="2" t="inlineStr">
         <is>
-          <t>“If you opt-in to receive newsletters, announcements, or advertisements of any kind from our business partners, we may share your Personal Information with such third parties, so that they can directly contact you regarding such offers. You may opt-out of any marketing offers from us or our business partners by informing us during your account sign-up process or through communications to us via email at [EMAIL]. Your opt-out does not apply to communications from [NAME] regarding any changes or updates to your account, or the non-marketing use of your Personal Information as described elsewhere in this Privacy Policy.”</t>
+          <t>[removed: notice text is kept for research only]</t>
         </is>
       </c>
       <c r="H64" s="2" t="inlineStr">
@@ -3728,7 +3728,7 @@
       </c>
       <c r="G65" s="2" t="inlineStr">
         <is>
-          <t>“You may review, correct, update, or delete your Personal Information maintained by us. Please provide us with sufficient proof of your identity and appropriate documentation of corrections to be made. You can contact us at: [EMAIL]”</t>
+          <t>[removed: notice text is kept for research only]</t>
         </is>
       </c>
       <c r="H65" s="2" t="inlineStr">
@@ -3776,7 +3776,7 @@
       </c>
       <c r="G66" s="2" t="inlineStr">
         <is>
-          <t>no matching text found</t>
+          <t>[removed: notice text is kept for research only]</t>
         </is>
       </c>
       <c r="H66" s="2" t="inlineStr"/>
@@ -3820,7 +3820,7 @@
       </c>
       <c r="G67" s="2" t="inlineStr">
         <is>
-          <t>(whole notice) The notice text is in English.</t>
+          <t>[removed: notice text is kept for research only]</t>
         </is>
       </c>
       <c r="H67" s="2" t="inlineStr">
@@ -3868,7 +3868,7 @@
       </c>
       <c r="G68" s="2" t="inlineStr">
         <is>
-          <t>“Please contact us at email address: [EMAIL], If you have any questions or comments regarding this Privacy Policy.”</t>
+          <t>[removed: notice text is kept for research only]</t>
         </is>
       </c>
       <c r="H68" s="2" t="inlineStr">
@@ -3916,7 +3916,7 @@
       </c>
       <c r="G69" s="2" t="inlineStr">
         <is>
-          <t>no matching text found</t>
+          <t>[removed: notice text is kept for research only]</t>
         </is>
       </c>
       <c r="H69" s="2" t="inlineStr"/>
@@ -3960,7 +3960,7 @@
       </c>
       <c r="G70" s="2" t="inlineStr">
         <is>
-          <t>no matching text found</t>
+          <t>[removed: notice text is kept for research only]</t>
         </is>
       </c>
       <c r="H70" s="2" t="inlineStr"/>
@@ -4004,7 +4004,7 @@
       </c>
       <c r="G71" s="2" t="inlineStr">
         <is>
-          <t>“This Privacy Policy applies to the website [URL] and other websites associated with such URL (collectively the “Website”) operated by [NAME]. By using the Website, you consent to the practices described herein. We may update this Privacy Policy from time to time to reflect Schools and its users feedback. You should periodically review this Privacy Policy to stay informed of our practices. Your continued use of the Website following any changes to this Privacy Policy constitutes your acceptance of those changes.”</t>
+          <t>[removed: notice text is kept for research only]</t>
         </is>
       </c>
       <c r="H71" s="2" t="inlineStr">
@@ -4052,7 +4052,7 @@
       </c>
       <c r="G72" s="2" t="inlineStr">
         <is>
-          <t>no matching text found</t>
+          <t>[removed: notice text is kept for research only]</t>
         </is>
       </c>
       <c r="H72" s="2" t="inlineStr"/>
@@ -4096,7 +4096,7 @@
       </c>
       <c r="G73" s="2" t="inlineStr">
         <is>
-          <t>no matching text found</t>
+          <t>[removed: notice text is kept for research only]</t>
         </is>
       </c>
       <c r="H73" s="2" t="inlineStr"/>
@@ -4140,7 +4140,7 @@
       </c>
       <c r="G74" s="2" t="inlineStr">
         <is>
-          <t>no matching text found</t>
+          <t>[removed: notice text is kept for research only]</t>
         </is>
       </c>
       <c r="H74" s="2" t="inlineStr"/>
@@ -4184,7 +4184,7 @@
       </c>
       <c r="G75" s="2" t="inlineStr">
         <is>
-          <t>no matching text found</t>
+          <t>[removed: notice text is kept for research only]</t>
         </is>
       </c>
       <c r="H75" s="2" t="inlineStr"/>
@@ -4228,7 +4228,7 @@
       </c>
       <c r="G76" s="2" t="inlineStr">
         <is>
-          <t>Closest text found (not necessarily enough for 'met'): “We may use third parties to better understand your user preferences and deliver targeted advertisements to you. These third parties may also place cookies on your computer. This policy does not apply to, and [NAME] is not responsible for, cookies placed or data collected by such third parties.”</t>
+          <t>[removed: notice text is kept for research only]</t>
         </is>
       </c>
       <c r="H76" s="2" t="inlineStr">
@@ -4276,7 +4276,7 @@
       </c>
       <c r="G77" s="2" t="inlineStr">
         <is>
-          <t>“When a student is admitted in our schools, we gather student name, parents details email, mobile number, address, name of previous school etc. Since, teachers have to prepare result and report card, they are going to use”</t>
+          <t>[removed: notice text is kept for research only]</t>
         </is>
       </c>
       <c r="H77" s="2" t="inlineStr">
@@ -4324,7 +4324,7 @@
       </c>
       <c r="G78" s="2" t="inlineStr">
         <is>
-          <t>“When a student is admitted in our schools, we gather student name, parents details email, mobile number, address, name of previous school etc. Since, teachers have to prepare result and report card, they are going to use these information. These information will be collected only to show them on report cards and We do not use your email id or students email id for sending unnecessary message or for promotion of any product. It will be used only for official communication.”</t>
+          <t>[removed: notice text is kept for research only]</t>
         </is>
       </c>
       <c r="H78" s="2" t="inlineStr">
@@ -4372,7 +4372,7 @@
       </c>
       <c r="G79" s="2" t="inlineStr">
         <is>
-          <t>no matching text found</t>
+          <t>[removed: notice text is kept for research only]</t>
         </is>
       </c>
       <c r="H79" s="2" t="inlineStr"/>
@@ -4416,7 +4416,7 @@
       </c>
       <c r="G80" s="2" t="inlineStr">
         <is>
-          <t>Closest text found (not necessarily enough for 'met'): “not to use for any unlawful activities. If you feel that the information provided by you about yourself and about students are sensitive in nature and may be misused by us or any other party, kindly do not provide such information.”</t>
+          <t>[removed: notice text is kept for research only]</t>
         </is>
       </c>
       <c r="H80" s="2" t="inlineStr">
@@ -4464,7 +4464,7 @@
       </c>
       <c r="G81" s="2" t="inlineStr">
         <is>
-          <t>no matching text found</t>
+          <t>[removed: notice text is kept for research only]</t>
         </is>
       </c>
       <c r="H81" s="2" t="inlineStr"/>
@@ -4508,7 +4508,7 @@
       </c>
       <c r="G82" s="2" t="inlineStr">
         <is>
-          <t>(whole notice) The notice text is in English.</t>
+          <t>[removed: notice text is kept for research only]</t>
         </is>
       </c>
       <c r="H82" s="2" t="inlineStr">
@@ -4556,7 +4556,7 @@
       </c>
       <c r="G83" s="2" t="inlineStr">
         <is>
-          <t>“[EMAIL] [PHONE]”  [page header of the website, not in the notice body]</t>
+          <t>[removed: notice text is kept for research only]</t>
         </is>
       </c>
       <c r="H83" s="2" t="inlineStr">
@@ -4604,7 +4604,7 @@
       </c>
       <c r="G84" s="2" t="inlineStr">
         <is>
-          <t>no matching text found</t>
+          <t>[removed: notice text is kept for research only]</t>
         </is>
       </c>
       <c r="H84" s="2" t="inlineStr"/>
@@ -4648,7 +4648,7 @@
       </c>
       <c r="G85" s="2" t="inlineStr">
         <is>
-          <t>no matching text found</t>
+          <t>[removed: notice text is kept for research only]</t>
         </is>
       </c>
       <c r="H85" s="2" t="inlineStr"/>
@@ -4692,7 +4692,7 @@
       </c>
       <c r="G86" s="2" t="inlineStr">
         <is>
-          <t>“knows that you care how information about you is used and shared and we appreciate your trust in us to do that carefully and sensibly. This notice describes our privacy policy. By visiting this website and using the our web applications, you are accepting and consenting to the practices described in this”</t>
+          <t>[removed: notice text is kept for research only]</t>
         </is>
       </c>
       <c r="H86" s="2" t="inlineStr">
@@ -4740,7 +4740,7 @@
       </c>
       <c r="G87" s="2" t="inlineStr">
         <is>
-          <t>Closest text found (not necessarily enough for 'met'): “When a student is admitted in our schools, we gather student name, parents details email, mobile number,”</t>
+          <t>[removed: notice text is kept for research only]</t>
         </is>
       </c>
       <c r="H87" s="2" t="inlineStr">
@@ -4788,7 +4788,7 @@
       </c>
       <c r="G88" s="2" t="inlineStr">
         <is>
-          <t>no matching text found</t>
+          <t>[removed: notice text is kept for research only]</t>
         </is>
       </c>
       <c r="H88" s="2" t="inlineStr"/>
@@ -4832,7 +4832,7 @@
       </c>
       <c r="G89" s="2" t="inlineStr">
         <is>
-          <t>no matching text found</t>
+          <t>[removed: notice text is kept for research only]</t>
         </is>
       </c>
       <c r="H89" s="2" t="inlineStr"/>
@@ -4876,7 +4876,7 @@
       </c>
       <c r="G90" s="2" t="inlineStr">
         <is>
-          <t>no matching text found</t>
+          <t>[removed: notice text is kept for research only]</t>
         </is>
       </c>
       <c r="H90" s="2" t="inlineStr"/>
@@ -4920,7 +4920,7 @@
       </c>
       <c r="G91" s="2" t="inlineStr">
         <is>
-          <t>Closest text found (not necessarily enough for 'met'): “Our site may include third-party advertising and links to other websites. Be careful when you decide to visit those websites shown as advertisement. We will not be”</t>
+          <t>[removed: notice text is kept for research only]</t>
         </is>
       </c>
       <c r="H91" s="2" t="inlineStr">
@@ -4968,7 +4968,7 @@
       </c>
       <c r="G92" s="2" t="inlineStr">
         <is>
-          <t>“When visitors leave comments on the site we collect the data shown in the comments form, and also the visitor’s IP address and browser user agent string to help spam detection. If you leave a comment on our site you may opt-in to saving your name, email address and website in cookies. These are for your convenience so that you do not have to fill in your details again when you leave another comment. These cookies will last for one year.”</t>
+          <t>[removed: notice text is kept for research only]</t>
         </is>
       </c>
       <c r="H92" s="2" t="inlineStr">
@@ -5016,7 +5016,7 @@
       </c>
       <c r="G93" s="2" t="inlineStr">
         <is>
-          <t>“When visitors leave comments on the site we collect the data shown in the comments form, and also the visitor’s IP address and browser user agent string to help spam detection. If you leave a comment on our site you may opt-in to saving your name, email address and website in cookies. These are for your convenience so that you do not have to fill in your details again when you leave another comment. These cookies will last for one year.”</t>
+          <t>[removed: notice text is kept for research only]</t>
         </is>
       </c>
       <c r="H93" s="2" t="inlineStr">
@@ -5064,7 +5064,7 @@
       </c>
       <c r="G94" s="2" t="inlineStr">
         <is>
-          <t>no matching text found</t>
+          <t>[removed: notice text is kept for research only]</t>
         </is>
       </c>
       <c r="H94" s="2" t="inlineStr"/>
@@ -5108,7 +5108,7 @@
       </c>
       <c r="G95" s="2" t="inlineStr">
         <is>
-          <t>“If you have an account on this site, or have left comments, you can request to receive an exported file of the personal data we hold about you, including any data you have provided to us. You can also request that we erase any personal data we hold about you. This does not include any data we are obliged to keep for administrative, legal, or security purposes.”</t>
+          <t>[removed: notice text is kept for research only]</t>
         </is>
       </c>
       <c r="H95" s="2" t="inlineStr">
@@ -5160,7 +5160,7 @@
       </c>
       <c r="G96" s="2" t="inlineStr">
         <is>
-          <t>no matching text found</t>
+          <t>[removed: notice text is kept for research only]</t>
         </is>
       </c>
       <c r="H96" s="2" t="inlineStr"/>
@@ -5204,7 +5204,7 @@
       </c>
       <c r="G97" s="2" t="inlineStr">
         <is>
-          <t>(whole notice) The notice text is in English.</t>
+          <t>[removed: notice text is kept for research only]</t>
         </is>
       </c>
       <c r="H97" s="2" t="inlineStr">
@@ -5252,7 +5252,7 @@
       </c>
       <c r="G98" s="2" t="inlineStr">
         <is>
-          <t>no matching text found</t>
+          <t>[removed: notice text is kept for research only]</t>
         </is>
       </c>
       <c r="H98" s="2" t="inlineStr"/>
@@ -5296,7 +5296,7 @@
       </c>
       <c r="G99" s="2" t="inlineStr">
         <is>
-          <t>no matching text found</t>
+          <t>[removed: notice text is kept for research only]</t>
         </is>
       </c>
       <c r="H99" s="2" t="inlineStr"/>
@@ -5340,7 +5340,7 @@
       </c>
       <c r="G100" s="2" t="inlineStr">
         <is>
-          <t>no matching text found</t>
+          <t>[removed: notice text is kept for research only]</t>
         </is>
       </c>
       <c r="H100" s="2" t="inlineStr"/>
@@ -5384,7 +5384,7 @@
       </c>
       <c r="G101" s="2" t="inlineStr">
         <is>
-          <t>“Who we are Suggested text: Our website address is: [URL]”</t>
+          <t>[removed: notice text is kept for research only]</t>
         </is>
       </c>
       <c r="H101" s="2" t="inlineStr">
@@ -5432,7 +5432,7 @@
       </c>
       <c r="G102" s="2" t="inlineStr">
         <is>
-          <t>no matching text found</t>
+          <t>[removed: notice text is kept for research only]</t>
         </is>
       </c>
       <c r="H102" s="2" t="inlineStr"/>
@@ -5476,7 +5476,7 @@
       </c>
       <c r="G103" s="2" t="inlineStr">
         <is>
-          <t>no matching text found</t>
+          <t>[removed: notice text is kept for research only]</t>
         </is>
       </c>
       <c r="H103" s="2" t="inlineStr"/>
@@ -5520,7 +5520,7 @@
       </c>
       <c r="G104" s="2" t="inlineStr">
         <is>
-          <t>no matching text found</t>
+          <t>[removed: notice text is kept for research only]</t>
         </is>
       </c>
       <c r="H104" s="2" t="inlineStr"/>
@@ -5564,7 +5564,7 @@
       </c>
       <c r="G105" s="2" t="inlineStr">
         <is>
-          <t>no matching text found</t>
+          <t>[removed: notice text is kept for research only]</t>
         </is>
       </c>
       <c r="H105" s="2" t="inlineStr"/>
@@ -5608,7 +5608,7 @@
       </c>
       <c r="G106" s="2" t="inlineStr">
         <is>
-          <t>Closest text found (not necessarily enough for 'met'): “Articles on this site may include embedded content (e.g. videos, images, articles, etc.). Embedded content from other websites behaves in the exact same way as if the visitor has visited the other website. These websites may collect data about you, use cookies, embed additional third-party tracking, and monitor your interaction with that embedded content, including tracking your interaction with the embedded content if you have an account and are logged in to that website.”</t>
+          <t>[removed: notice text is kept for research only]</t>
         </is>
       </c>
       <c r="H106" s="2" t="inlineStr">
@@ -5656,7 +5656,7 @@
       </c>
       <c r="G107" s="2" t="inlineStr">
         <is>
-          <t>“Personal Information: This includes information that can be used to identify you, such as your name, email address, phone number, physical address, student ID number, and academic information. Demographic Information: This includes information about your age, gender, location, and interests. Usage Information: This includes information about your use of the Website, such as the pages you visit, the links you click, and the time you spend on the Website. Device Information: This includes information about your device, such as your browser type, operating system, and IP address.”</t>
+          <t>[removed: notice text is kept for research only]</t>
         </is>
       </c>
       <c r="H107" s="2" t="inlineStr">
@@ -5704,7 +5704,7 @@
       </c>
       <c r="G108" s="2" t="inlineStr">
         <is>
-          <t>“We use your information for the following purposes: To provide and improve the Website and our services. To personalize your experience on the Website. To send you important information about the Website and our services. To provide you with customer support. To comply with legal and regulatory requirements.”</t>
+          <t>[removed: notice text is kept for research only]</t>
         </is>
       </c>
       <c r="H108" s="2" t="inlineStr">
@@ -5752,7 +5752,7 @@
       </c>
       <c r="G109" s="2" t="inlineStr">
         <is>
-          <t>“You have the following choices regarding your information: You can unsubscribe from our marketing emails by clicking on the "unsubscribe" link in any email we send you. You can opt out of the collection of your information by using the settings in your browser.”</t>
+          <t>[removed: notice text is kept for research only]</t>
         </is>
       </c>
       <c r="H109" s="2" t="inlineStr">
@@ -5800,7 +5800,7 @@
       </c>
       <c r="G110" s="2" t="inlineStr">
         <is>
-          <t>“Please write to or email us as soon as you can, if you think that any information we are holding on you is inaccurate or incomplete. If any information is discovered to be inaccurate, it will be updated right away.”</t>
+          <t>[removed: notice text is kept for research only]</t>
         </is>
       </c>
       <c r="H110" s="2" t="inlineStr">
@@ -5848,7 +5848,7 @@
       </c>
       <c r="G111" s="2" t="inlineStr">
         <is>
-          <t>no matching text found</t>
+          <t>[removed: notice text is kept for research only]</t>
         </is>
       </c>
       <c r="H111" s="2" t="inlineStr"/>
@@ -5892,7 +5892,7 @@
       </c>
       <c r="G112" s="2" t="inlineStr">
         <is>
-          <t>(whole notice) The notice text is in English.</t>
+          <t>[removed: notice text is kept for research only]</t>
         </is>
       </c>
       <c r="H112" s="2" t="inlineStr">
@@ -5940,7 +5940,7 @@
       </c>
       <c r="G113" s="2" t="inlineStr">
         <is>
-          <t>“If you have any questions about this Privacy Policy, please contact us by email.”</t>
+          <t>[removed: notice text is kept for research only]</t>
         </is>
       </c>
       <c r="H113" s="2" t="inlineStr">
@@ -5988,7 +5988,7 @@
       </c>
       <c r="G114" s="2" t="inlineStr">
         <is>
-          <t>no matching text found</t>
+          <t>[removed: notice text is kept for research only]</t>
         </is>
       </c>
       <c r="H114" s="2" t="inlineStr"/>
@@ -6032,7 +6032,7 @@
       </c>
       <c r="G115" s="2" t="inlineStr">
         <is>
-          <t>no matching text found</t>
+          <t>[removed: notice text is kept for research only]</t>
         </is>
       </c>
       <c r="H115" s="2" t="inlineStr"/>
@@ -6076,7 +6076,7 @@
       </c>
       <c r="G116" s="2" t="inlineStr">
         <is>
-          <t>“[NAME] ("[NAME]", "we", "us", or "our") is committed to protecting the privacy of our users ("you" or "your"). This Privacy Policy explains how we collect, use, and disclose information that we may collect from you when you visit our website ("Website").”</t>
+          <t>[removed: notice text is kept for research only]</t>
         </is>
       </c>
       <c r="H116" s="2" t="inlineStr">
@@ -6124,7 +6124,7 @@
       </c>
       <c r="G117" s="2" t="inlineStr">
         <is>
-          <t>no matching text found</t>
+          <t>[removed: notice text is kept for research only]</t>
         </is>
       </c>
       <c r="H117" s="2" t="inlineStr"/>
@@ -6168,7 +6168,7 @@
       </c>
       <c r="G118" s="2" t="inlineStr">
         <is>
-          <t>no matching text found</t>
+          <t>[removed: notice text is kept for research only]</t>
         </is>
       </c>
       <c r="H118" s="2" t="inlineStr"/>
@@ -6212,7 +6212,7 @@
       </c>
       <c r="G119" s="2" t="inlineStr">
         <is>
-          <t>no matching text found</t>
+          <t>[removed: notice text is kept for research only]</t>
         </is>
       </c>
       <c r="H119" s="2" t="inlineStr"/>
@@ -6256,7 +6256,7 @@
       </c>
       <c r="G120" s="2" t="inlineStr">
         <is>
-          <t>no matching text found</t>
+          <t>[removed: notice text is kept for research only]</t>
         </is>
       </c>
       <c r="H120" s="2" t="inlineStr"/>
@@ -6300,7 +6300,7 @@
       </c>
       <c r="G121" s="2" t="inlineStr">
         <is>
-          <t>Closest text found (not necessarily enough for 'met'): “We use cookies and similar technologies to track the activity on our Website and hold certain information. Cookies are files with small amount of data that may include an anonymous unique identifier. Cookies are sent to your browser from a website and stored on your device. Tracking technologies used are also beacons, tags, and scripts to collect and analyze information and improve your experience on our Website.”</t>
+          <t>[removed: notice text is kept for research only]</t>
         </is>
       </c>
       <c r="H121" s="2" t="inlineStr">
@@ -6348,7 +6348,7 @@
       </c>
       <c r="G122" s="2" t="inlineStr">
         <is>
-          <t>“We collect certain data from you directly, like information you enter yourself, data about your participation in courses, and data from third-party platforms you connect with eCademy . We also collect some data automatically, like information about your device and what parts of our Services you interact with or spend time using. 2. Data You Provide to Us We may collect different data from or about you depending on how you use the Services. Below are some examples to help you better understand the data we collect.”  [the 'examples' list is missing from the extracted text (collapsed content on the page)]</t>
+          <t>[removed: notice text is kept for research only]</t>
         </is>
       </c>
       <c r="H122" s="2" t="inlineStr">
@@ -6396,7 +6396,7 @@
       </c>
       <c r="G123" s="2" t="inlineStr">
         <is>
-          <t>“4. For What We Use Your Data Responding to your questions and concerns; Sending you administrative messages and information, including messages from instructors and teaching assistants, notifications about changes to our Service, and updates to our agreements; Sending push notifications to your wireless device to provide updates and other relevant messages (which you can manage from the “options” or “settings” page of the mobile app);”</t>
+          <t>[removed: notice text is kept for research only]</t>
         </is>
       </c>
       <c r="H123" s="2" t="inlineStr">
@@ -6444,7 +6444,7 @@
       </c>
       <c r="G124" s="2" t="inlineStr">
         <is>
-          <t>“To stop receiving promotional communications from us, you can opt out by using the unsubscribe mechanism in the promotional communication you receive or by changing the email preferences in your account. Note that regardless of your email preference settings, we will send you transactional and relationship messages regarding the Services, including administrative confirmations, order confirmations, important updates about the Services, and notices about our policies.”</t>
+          <t>[removed: notice text is kept for research only]</t>
         </is>
       </c>
       <c r="H124" s="2" t="inlineStr">
@@ -6492,7 +6492,7 @@
       </c>
       <c r="G125" s="2" t="inlineStr">
         <is>
-          <t>“To update data you provide directly, log into your account and update your account at any time.”</t>
+          <t>[removed: notice text is kept for research only]</t>
         </is>
       </c>
       <c r="H125" s="2" t="inlineStr">
@@ -6540,7 +6540,7 @@
       </c>
       <c r="G126" s="2" t="inlineStr">
         <is>
-          <t>no matching text found</t>
+          <t>[removed: notice text is kept for research only]</t>
         </is>
       </c>
       <c r="H126" s="2" t="inlineStr"/>
@@ -6584,7 +6584,7 @@
       </c>
       <c r="G127" s="2" t="inlineStr">
         <is>
-          <t>(whole notice) The notice text is in English.</t>
+          <t>[removed: notice text is kept for research only]</t>
         </is>
       </c>
       <c r="H127" s="2" t="inlineStr">
@@ -6632,7 +6632,7 @@
       </c>
       <c r="G128" s="2" t="inlineStr">
         <is>
-          <t>Closest text found (not necessarily enough for 'met'): “[EMAIL]”  [page header of the website only]</t>
+          <t>[removed: notice text is kept for research only]</t>
         </is>
       </c>
       <c r="H128" s="2" t="inlineStr">
@@ -6688,7 +6688,7 @@
       </c>
       <c r="G129" s="2" t="inlineStr">
         <is>
-          <t>no matching text found</t>
+          <t>[removed: notice text is kept for research only]</t>
         </is>
       </c>
       <c r="H129" s="2" t="inlineStr"/>
@@ -6732,7 +6732,7 @@
       </c>
       <c r="G130" s="2" t="inlineStr">
         <is>
-          <t>no matching text found</t>
+          <t>[removed: notice text is kept for research only]</t>
         </is>
       </c>
       <c r="H130" s="2" t="inlineStr"/>
@@ -6776,7 +6776,7 @@
       </c>
       <c r="G131" s="2" t="inlineStr">
         <is>
-          <t>“This Privacy Policy was last updated on January 1, 2020. 1. What Data We Get”</t>
+          <t>[removed: notice text is kept for research only]</t>
         </is>
       </c>
       <c r="H131" s="2" t="inlineStr">
@@ -6824,7 +6824,7 @@
       </c>
       <c r="G132" s="2" t="inlineStr">
         <is>
-          <t>“6. Our Policy Concerning Children We recognize the privacy interests of children and encourage parents and guardians to take an active role in their children’s online activities and interests. Children under 13 (or under 16 in the European Economic Area) should not use the Services. If we learn that we’ve collected personal data from a child under those ages, we will take reasonable steps to delete it.”</t>
+          <t>[removed: notice text is kept for research only]</t>
         </is>
       </c>
       <c r="H132" s="2" t="inlineStr">
@@ -6872,7 +6872,7 @@
       </c>
       <c r="G133" s="2" t="inlineStr">
         <is>
-          <t>“We recognize the privacy interests of children and encourage parents and guardians to take an active role in their children’s online activities and interests. Children under 13 (or under 16 in the European Economic Area) should not use the Services. If we learn that we’ve collected personal data from a child under those ages, we will take reasonable steps to delete it.”</t>
+          <t>[removed: notice text is kept for research only]</t>
         </is>
       </c>
       <c r="H133" s="2" t="inlineStr">
@@ -6920,7 +6920,7 @@
       </c>
       <c r="G134" s="2" t="inlineStr">
         <is>
-          <t>Closest text found (not necessarily enough for 'met'): “We recognize the privacy interests of children and encourage parents and guardians to take an active role in their children’s online activities and interests. Children under 13 (or under 16 in the European Economic Area) should not use the Services. If we learn that we’ve collected personal data from a child under those ages, we will take reasonable steps to delete it.”</t>
+          <t>[removed: notice text is kept for research only]</t>
         </is>
       </c>
       <c r="H134" s="2" t="inlineStr">
@@ -6968,7 +6968,7 @@
       </c>
       <c r="G135" s="2" t="inlineStr">
         <is>
-          <t>no matching text found</t>
+          <t>[removed: notice text is kept for research only]</t>
         </is>
       </c>
       <c r="H135" s="2" t="inlineStr"/>
@@ -7012,7 +7012,7 @@
       </c>
       <c r="G136" s="2" t="inlineStr">
         <is>
-          <t>Closest text found (not necessarily enough for 'met'): “We use tools like cookies, web beacons, analytics services, and advertising providers to gather the data listed above. Some of these tools offer you the ability to opt out of data collection. To get information and control cookies used for tailored advertising from participating companies, see the consumer opt-out pages for the Network Advertising Initiative and Digital Advertising Alliance, or if you’re located in the European Union, visit the Your Online Choices site. To opt out of Google’s display advertising or customize Google Display Network ads, visit the Google Ads Settings page. To opt out of Taboola’s targeted ads, see the Opt-out Link in their Cookie Policy.”</t>
+          <t>[removed: notice text is kept for research only]</t>
         </is>
       </c>
       <c r="H136" s="2" t="inlineStr">
@@ -7060,7 +7060,7 @@
       </c>
       <c r="G137" s="2" t="inlineStr">
         <is>
-          <t>“[NAME] may collect the following information from its users: Information you provide to us: You may choose to disclose information including your name, email, address and any additional information. Information that is automatically collected: When you visit the [NAME] Website, we may automatically collect non-personally identifiable information, such as information about your hardware devices, your use of the website, and information about the website that referred you to the site.”</t>
+          <t>[removed: notice text is kept for research only]</t>
         </is>
       </c>
       <c r="H137" s="2" t="inlineStr">
@@ -7108,7 +7108,7 @@
       </c>
       <c r="G138" s="2" t="inlineStr">
         <is>
-          <t>“By providing your name, address and any additional information, you freely consent to [NAME] holding, using and processing your personal data for the purposes set out by the nature of our business and on this website and where necessary. It may also be utilized for the purposes of assessing your potential needs, for marketing research and for marketing to you of services catered by the [NAME].”</t>
+          <t>[removed: notice text is kept for research only]</t>
         </is>
       </c>
       <c r="H138" s="2" t="inlineStr">
@@ -7156,7 +7156,7 @@
       </c>
       <c r="G139" s="2" t="inlineStr">
         <is>
-          <t>Closest text found (not necessarily enough for 'met'): “Should the roles for which [NAME] holds, uses or processes your personal information change in any direction, you will be advised of such modifications by means of a notice posted on this page so that you are always mindful of what information we gather, how we use it, and under what circumstances we reveal it. At that time you will be granted the chance to refuse to have your personal data held, used or processed for such changed purposes. You agree to accept notification in this manner if you post any data through this website.”</t>
+          <t>[removed: notice text is kept for research only]</t>
         </is>
       </c>
       <c r="H139" s="2" t="inlineStr">
@@ -7204,7 +7204,7 @@
       </c>
       <c r="G140" s="2" t="inlineStr">
         <is>
-          <t>“If for whatever reason, you are concerned that the personal information maintained at [NAME] is not correct or have any queries about privacy policies, please contact us at [EMAIL].”</t>
+          <t>[removed: notice text is kept for research only]</t>
         </is>
       </c>
       <c r="H140" s="2" t="inlineStr">
@@ -7252,7 +7252,7 @@
       </c>
       <c r="G141" s="2" t="inlineStr">
         <is>
-          <t>no matching text found</t>
+          <t>[removed: notice text is kept for research only]</t>
         </is>
       </c>
       <c r="H141" s="2" t="inlineStr"/>
@@ -7296,7 +7296,7 @@
       </c>
       <c r="G142" s="2" t="inlineStr">
         <is>
-          <t>(whole notice) The notice text is in English.</t>
+          <t>[removed: notice text is kept for research only]</t>
         </is>
       </c>
       <c r="H142" s="2" t="inlineStr">
@@ -7344,7 +7344,7 @@
       </c>
       <c r="G143" s="2" t="inlineStr">
         <is>
-          <t>“If for whatever reason, you are concerned that the personal information maintained at [NAME] is not correct or have any queries about privacy policies, please contact us at [EMAIL].”</t>
+          <t>[removed: notice text is kept for research only]</t>
         </is>
       </c>
       <c r="H143" s="2" t="inlineStr">
@@ -7392,7 +7392,7 @@
       </c>
       <c r="G144" s="2" t="inlineStr">
         <is>
-          <t>no matching text found</t>
+          <t>[removed: notice text is kept for research only]</t>
         </is>
       </c>
       <c r="H144" s="2" t="inlineStr"/>
@@ -7436,7 +7436,7 @@
       </c>
       <c r="G145" s="2" t="inlineStr">
         <is>
-          <t>no matching text found</t>
+          <t>[removed: notice text is kept for research only]</t>
         </is>
       </c>
       <c r="H145" s="2" t="inlineStr"/>
@@ -7480,7 +7480,7 @@
       </c>
       <c r="G146" s="2" t="inlineStr">
         <is>
-          <t>“[NAME] would like all users of our website to know that we are concerned about your privacy and the security of any personal data that you may supply to us through this web site.”</t>
+          <t>[removed: notice text is kept for research only]</t>
         </is>
       </c>
       <c r="H146" s="2" t="inlineStr">
@@ -7528,7 +7528,7 @@
       </c>
       <c r="G147" s="2" t="inlineStr">
         <is>
-          <t>no matching text found</t>
+          <t>[removed: notice text is kept for research only]</t>
         </is>
       </c>
       <c r="H147" s="2" t="inlineStr"/>
@@ -7572,7 +7572,7 @@
       </c>
       <c r="G148" s="2" t="inlineStr">
         <is>
-          <t>no matching text found</t>
+          <t>[removed: notice text is kept for research only]</t>
         </is>
       </c>
       <c r="H148" s="2" t="inlineStr"/>
@@ -7616,7 +7616,7 @@
       </c>
       <c r="G149" s="2" t="inlineStr">
         <is>
-          <t>no matching text found</t>
+          <t>[removed: notice text is kept for research only]</t>
         </is>
       </c>
       <c r="H149" s="2" t="inlineStr"/>
@@ -7660,7 +7660,7 @@
       </c>
       <c r="G150" s="2" t="inlineStr">
         <is>
-          <t>no matching text found</t>
+          <t>[removed: notice text is kept for research only]</t>
         </is>
       </c>
       <c r="H150" s="2" t="inlineStr"/>
@@ -7704,7 +7704,7 @@
       </c>
       <c r="G151" s="2" t="inlineStr">
         <is>
-          <t>Closest text found (not necessarily enough for 'met'): “When you visit the [NAME] Website, we may automatically collect non-personally identifiable information, such as information about your hardware devices, your use of the website, and information about the website that referred you to the site. [NAME] may combine information provided by you with information from third parties, for the purpose of providing you better service. Examples of such information include address verification service or data analytics.”</t>
+          <t>[removed: notice text is kept for research only]</t>
         </is>
       </c>
       <c r="H151" s="2" t="inlineStr">
@@ -7752,7 +7752,7 @@
       </c>
       <c r="G152" s="2" t="inlineStr">
         <is>
-          <t>“We collect information from you when you interact with our website, including: Personal Information: Name, email address, phone number, address, and other contact details provided by you in forms, such as admission or inquiry forms. Usage Information: Information about how you use our website, such as IP address, browser type, and pages visited.”</t>
+          <t>[removed: notice text is kept for research only]</t>
         </is>
       </c>
       <c r="H152" s="2" t="inlineStr">
@@ -7800,7 +7800,7 @@
       </c>
       <c r="G153" s="2" t="inlineStr">
         <is>
-          <t>“2. How We Use Your Information We use the information we collect for purposes such as: Communication: To respond to inquiries, process applications, and provide updates or news about the school. Improvement: To improve our website, services, and student experience. Compliance: To comply with legal obligations and protect the safety of our students, staff, and community.”</t>
+          <t>[removed: notice text is kept for research only]</t>
         </is>
       </c>
       <c r="H153" s="2" t="inlineStr">
@@ -7848,7 +7848,7 @@
       </c>
       <c r="G154" s="2" t="inlineStr">
         <is>
-          <t>“Opt out of receiving communications by following the instructions in our emails.”</t>
+          <t>[removed: notice text is kept for research only]</t>
         </is>
       </c>
       <c r="H154" s="2" t="inlineStr">
@@ -7896,7 +7896,7 @@
       </c>
       <c r="G155" s="2" t="inlineStr">
         <is>
-          <t>Closest text found (not necessarily enough for 'met'): “Opt out of receiving communications by following the instructions in our emails. Disable cookies via your browser settings, though this may impact site functionality.”</t>
+          <t>[removed: notice text is kept for research only]</t>
         </is>
       </c>
       <c r="H155" s="2" t="inlineStr">
@@ -7952,7 +7952,7 @@
       </c>
       <c r="G156" s="2" t="inlineStr">
         <is>
-          <t>no matching text found</t>
+          <t>[removed: notice text is kept for research only]</t>
         </is>
       </c>
       <c r="H156" s="2" t="inlineStr"/>
@@ -7996,7 +7996,7 @@
       </c>
       <c r="G157" s="2" t="inlineStr">
         <is>
-          <t>(whole notice) The notice text is in English.</t>
+          <t>[removed: notice text is kept for research only]</t>
         </is>
       </c>
       <c r="H157" s="2" t="inlineStr">
@@ -8044,7 +8044,7 @@
       </c>
       <c r="G158" s="2" t="inlineStr">
         <is>
-          <t>“If you have any questions or concerns about this Privacy Policy, please contact us at: Email: [EMAIL] Phone: [PHONE] / [PHONE]”</t>
+          <t>[removed: notice text is kept for research only]</t>
         </is>
       </c>
       <c r="H158" s="2" t="inlineStr">
@@ -8092,7 +8092,7 @@
       </c>
       <c r="G159" s="2" t="inlineStr">
         <is>
-          <t>no matching text found</t>
+          <t>[removed: notice text is kept for research only]</t>
         </is>
       </c>
       <c r="H159" s="2" t="inlineStr"/>
@@ -8136,7 +8136,7 @@
       </c>
       <c r="G160" s="2" t="inlineStr">
         <is>
-          <t>no matching text found</t>
+          <t>[removed: notice text is kept for research only]</t>
         </is>
       </c>
       <c r="H160" s="2" t="inlineStr"/>
@@ -8180,7 +8180,7 @@
       </c>
       <c r="G161" s="2" t="inlineStr">
         <is>
-          <t>“[NAME] (referred to as “we,” “us,” or “our”) respects the privacy of our students, parents, and website visitors. This Privacy Policy outlines how we collect, use, disclose, and safeguard your personal information when you visit our website,”</t>
+          <t>[removed: notice text is kept for research only]</t>
         </is>
       </c>
       <c r="H161" s="2" t="inlineStr">
@@ -8228,7 +8228,7 @@
       </c>
       <c r="G162" s="2" t="inlineStr">
         <is>
-          <t>Closest text found (not necessarily enough for 'met'): “[NAME] (referred to as “we,” “us,” or “our”) respects the privacy of our students, parents, and website visitors. This Privacy Policy outlines how we collect, use, disclose, and safeguard your personal information when you visit our website,”</t>
+          <t>[removed: notice text is kept for research only]</t>
         </is>
       </c>
       <c r="H162" s="2" t="inlineStr">
@@ -8276,7 +8276,7 @@
       </c>
       <c r="G163" s="2" t="inlineStr">
         <is>
-          <t>no matching text found</t>
+          <t>[removed: notice text is kept for research only]</t>
         </is>
       </c>
       <c r="H163" s="2" t="inlineStr"/>
@@ -8320,7 +8320,7 @@
       </c>
       <c r="G164" s="2" t="inlineStr">
         <is>
-          <t>no matching text found</t>
+          <t>[removed: notice text is kept for research only]</t>
         </is>
       </c>
       <c r="H164" s="2" t="inlineStr"/>
@@ -8364,7 +8364,7 @@
       </c>
       <c r="G165" s="2" t="inlineStr">
         <is>
-          <t>no matching text found</t>
+          <t>[removed: notice text is kept for research only]</t>
         </is>
       </c>
       <c r="H165" s="2" t="inlineStr"/>
@@ -8408,7 +8408,7 @@
       </c>
       <c r="G166" s="2" t="inlineStr">
         <is>
-          <t>Closest text found (not necessarily enough for 'met'): “Cookies and Tracking Technologies: We use cookies to enhance your experience, analyze usage, and improve our site.”</t>
+          <t>[removed: notice text is kept for research only]</t>
         </is>
       </c>
       <c r="H166" s="2" t="inlineStr">
@@ -8456,7 +8456,7 @@
       </c>
       <c r="G167" s="2" t="inlineStr">
         <is>
-          <t>“What information do we collect from you? We collect your personal information to provide and continuously enhance our services for all customers. This information is obtained when you visit our website and complete a form. When filling out a form, you may be required to enter details such as your name, email address, phone number, and any other necessary information. However, you have the option to visit our site anonymously.”</t>
+          <t>[removed: notice text is kept for research only]</t>
         </is>
       </c>
       <c r="H167" s="2" t="inlineStr">
@@ -8504,7 +8504,7 @@
       </c>
       <c r="G168" s="2" t="inlineStr">
         <is>
-          <t>“What do we use your information for? Any information collected from you may be used in one or all of the following ways: To personalise your experience (your information helps us better respond to your individual needs). To improve our website (we continually strive to enhance our website offerings based on the information and feedback we receive from you). To enhance customer service (your information helps us respond more effectively to service requests and support needs). To send periodic emails. The email address you provide for contact requests may be used to send you information and updates related to your request, in addition to occasional company news, updates, promotions, related products, or service information.”</t>
+          <t>[removed: notice text is kept for research only]</t>
         </is>
       </c>
       <c r="H168" s="2" t="inlineStr">
@@ -8552,7 +8552,7 @@
       </c>
       <c r="G169" s="2" t="inlineStr">
         <is>
-          <t>“If you wish to unsubscribe from future emails, simply respond to the received email indicating your preference, and we will promptly remove you from our database. Alternatively, follow the unsubscribe link enclosed within the email.”</t>
+          <t>[removed: notice text is kept for research only]</t>
         </is>
       </c>
       <c r="H169" s="2" t="inlineStr">
@@ -8600,7 +8600,7 @@
       </c>
       <c r="G170" s="2" t="inlineStr">
         <is>
-          <t>no matching text found</t>
+          <t>[removed: notice text is kept for research only]</t>
         </is>
       </c>
       <c r="H170" s="2" t="inlineStr"/>
@@ -8652,7 +8652,7 @@
       </c>
       <c r="G171" s="2" t="inlineStr">
         <is>
-          <t>no matching text found</t>
+          <t>[removed: notice text is kept for research only]</t>
         </is>
       </c>
       <c r="H171" s="2" t="inlineStr"/>
@@ -8696,7 +8696,7 @@
       </c>
       <c r="G172" s="2" t="inlineStr">
         <is>
-          <t>(whole notice) The notice text is in English.</t>
+          <t>[removed: notice text is kept for research only]</t>
         </is>
       </c>
       <c r="H172" s="2" t="inlineStr">
@@ -8744,7 +8744,7 @@
       </c>
       <c r="G173" s="2" t="inlineStr">
         <is>
-          <t>“If you have any questions or suggestions regarding this privacy policy, please feel free to contact us using the information below: Phone: [PHONE] Email: [EMAIL]”</t>
+          <t>[removed: notice text is kept for research only]</t>
         </is>
       </c>
       <c r="H173" s="2" t="inlineStr">
@@ -8792,7 +8792,7 @@
       </c>
       <c r="G174" s="2" t="inlineStr">
         <is>
-          <t>no matching text found</t>
+          <t>[removed: notice text is kept for research only]</t>
         </is>
       </c>
       <c r="H174" s="2" t="inlineStr"/>
@@ -8836,7 +8836,7 @@
       </c>
       <c r="G175" s="2" t="inlineStr">
         <is>
-          <t>no matching text found</t>
+          <t>[removed: notice text is kept for research only]</t>
         </is>
       </c>
       <c r="H175" s="2" t="inlineStr"/>
@@ -8880,7 +8880,7 @@
       </c>
       <c r="G176" s="2" t="inlineStr">
         <is>
-          <t>“This section helps you understand, how we at the [NAME] Foundation respect and safeguard your personal information that you submit whilst using our website. This Privacy Policy has been created for [NAME]”</t>
+          <t>[removed: notice text is kept for research only]</t>
         </is>
       </c>
       <c r="H176" s="2" t="inlineStr">
@@ -8928,7 +8928,7 @@
       </c>
       <c r="G177" s="2" t="inlineStr">
         <is>
-          <t>“You must be at least 18 years of age or the required legal age in your location to use our website or the resources contained therein. By using our website, you confirm that you are at least 18 years of age or the required legal age in your location and legally accept the terms and conditions of this”</t>
+          <t>[removed: notice text is kept for research only]</t>
         </is>
       </c>
       <c r="H177" s="2" t="inlineStr">
@@ -8976,7 +8976,7 @@
       </c>
       <c r="G178" s="2" t="inlineStr">
         <is>
-          <t>“You must be at least 18 years of age or the required legal age in your location to use our website or the resources contained therein. By using our website, you confirm that you are at least 18 years of age or the required legal age in your location and legally accept the terms and conditions of this”</t>
+          <t>[removed: notice text is kept for research only]</t>
         </is>
       </c>
       <c r="H178" s="2" t="inlineStr">
@@ -9024,7 +9024,7 @@
       </c>
       <c r="G179" s="2" t="inlineStr">
         <is>
-          <t>Closest text found (not necessarily enough for 'met'): “We pledge to you, our customer, that we have made a dedicated effort to align our privacy policy with the following important privacy laws and initiatives: Federal Trade Commission Fair California Online Privacy Protection Act Children’s Online Privacy Protection Act”</t>
+          <t>[removed: notice text is kept for research only]</t>
         </is>
       </c>
       <c r="H179" s="2" t="inlineStr">
@@ -9072,7 +9072,7 @@
       </c>
       <c r="G180" s="2" t="inlineStr">
         <is>
-          <t>no matching text found</t>
+          <t>[removed: notice text is kept for research only]</t>
         </is>
       </c>
       <c r="H180" s="2" t="inlineStr"/>
@@ -9116,7 +9116,7 @@
       </c>
       <c r="G181" s="2" t="inlineStr">
         <is>
-          <t>Closest text found (not necessarily enough for 'met'): “We do not sell, trade, share, or otherwise transfer your personally identifiable information to outside parties without your consent. However, this assurance does not include trusted third parties who assist us in operating our website, conducting our business, or servicing you, as long as those parties agree to keep this information confidential. We may also release your information when we believe that such release is appropriate to comply with the law, enforce our site policies, or protect our or others’ rights, property, or safety. However, non-personally identifiable visitor information may be provided to other parties for marketing, advertising, or other uses.”</t>
+          <t>[removed: notice text is kept for research only]</t>
         </is>
       </c>
       <c r="H181" s="2" t="inlineStr">
@@ -9164,7 +9164,7 @@
       </c>
       <c r="G182" s="2" t="inlineStr">
         <is>
-          <t>“We collect personal information to facilitate school operations and improve user experience. The data collected may include, but is not limited to: Names, contact details (phone numbers, email addresses), and academic records. Information provided during admissions, inquiries, or registration processes. Cookies and tracking technologies to improve website functionality and gather analytics. This may include IP addresses, browser types, and usage data.”</t>
+          <t>[removed: notice text is kept for research only]</t>
         </is>
       </c>
       <c r="H182" s="2" t="inlineStr">
@@ -9212,7 +9212,7 @@
       </c>
       <c r="G183" s="2" t="inlineStr">
         <is>
-          <t>“The data we collect is used to: Process admissions and maintain academic records. Communicate with students, parents, alumni, and staff. Improve our website’s functionality and performance through analytics tools such as Google Analytics, Google Search Console, and Cloudflare. Provide a secure and tailored browsing experience for users.”</t>
+          <t>[removed: notice text is kept for research only]</t>
         </is>
       </c>
       <c r="H183" s="2" t="inlineStr">
@@ -9260,7 +9260,7 @@
       </c>
       <c r="G184" s="2" t="inlineStr">
         <is>
-          <t>no matching text found</t>
+          <t>[removed: notice text is kept for research only]</t>
         </is>
       </c>
       <c r="H184" s="2" t="inlineStr"/>
@@ -9304,7 +9304,7 @@
       </c>
       <c r="G185" s="2" t="inlineStr">
         <is>
-          <t>“User Rights You have the right to: Access, update, or correct your personal information. Request deletion of your data, subject to legal and regulatory obligations. For minors (students), we ensure extra protection and require parental or guardian consent for data processing, where applicable.”</t>
+          <t>[removed: notice text is kept for research only]</t>
         </is>
       </c>
       <c r="H185" s="2" t="inlineStr">
@@ -9352,7 +9352,7 @@
       </c>
       <c r="G186" s="2" t="inlineStr">
         <is>
-          <t>no matching text found</t>
+          <t>[removed: notice text is kept for research only]</t>
         </is>
       </c>
       <c r="H186" s="2" t="inlineStr"/>
@@ -9396,7 +9396,7 @@
       </c>
       <c r="G187" s="2" t="inlineStr">
         <is>
-          <t>(whole notice) The notice text is in English.</t>
+          <t>[removed: notice text is kept for research only]</t>
         </is>
       </c>
       <c r="H187" s="2" t="inlineStr">
@@ -9444,7 +9444,7 @@
       </c>
       <c r="G188" s="2" t="inlineStr">
         <is>
-          <t>no matching text found</t>
+          <t>[removed: notice text is kept for research only]</t>
         </is>
       </c>
       <c r="H188" s="2" t="inlineStr"/>
@@ -9488,7 +9488,7 @@
       </c>
       <c r="G189" s="2" t="inlineStr">
         <is>
-          <t>no matching text found</t>
+          <t>[removed: notice text is kept for research only]</t>
         </is>
       </c>
       <c r="H189" s="2" t="inlineStr"/>
@@ -9532,7 +9532,7 @@
       </c>
       <c r="G190" s="2" t="inlineStr">
         <is>
-          <t>no matching text found</t>
+          <t>[removed: notice text is kept for research only]</t>
         </is>
       </c>
       <c r="H190" s="2" t="inlineStr"/>
@@ -9576,7 +9576,7 @@
       </c>
       <c r="G191" s="2" t="inlineStr">
         <is>
-          <t>“At [NAME], we are committed to protecting the privacy and personal information of our students, parents, alumni, and staff. This Privacy Policy explains how we collect, use, share, and protect your personal data in compliance with Indian privacy laws, including the Information Technology Act, 2000, and the Data Protection Rules, 2011.”</t>
+          <t>[removed: notice text is kept for research only]</t>
         </is>
       </c>
       <c r="H191" s="2" t="inlineStr">
@@ -9624,7 +9624,7 @@
       </c>
       <c r="G192" s="2" t="inlineStr">
         <is>
-          <t>“Request deletion of your data, subject to legal and regulatory obligations. For minors (students), we ensure extra protection and require parental or guardian consent for data processing, where applicable.”</t>
+          <t>[removed: notice text is kept for research only]</t>
         </is>
       </c>
       <c r="H192" s="2" t="inlineStr">
@@ -9672,7 +9672,7 @@
       </c>
       <c r="G193" s="2" t="inlineStr">
         <is>
-          <t>no matching text found</t>
+          <t>[removed: notice text is kept for research only]</t>
         </is>
       </c>
       <c r="H193" s="2" t="inlineStr"/>
@@ -9716,7 +9716,7 @@
       </c>
       <c r="G194" s="2" t="inlineStr">
         <is>
-          <t>“Request deletion of your data, subject to legal and regulatory obligations. For minors (students), we ensure extra protection and require parental or guardian consent for data processing, where applicable.”</t>
+          <t>[removed: notice text is kept for research only]</t>
         </is>
       </c>
       <c r="H194" s="2" t="inlineStr">
@@ -9764,7 +9764,7 @@
       </c>
       <c r="G195" s="2" t="inlineStr">
         <is>
-          <t>no matching text found</t>
+          <t>[removed: notice text is kept for research only]</t>
         </is>
       </c>
       <c r="H195" s="2" t="inlineStr"/>
@@ -9808,7 +9808,7 @@
       </c>
       <c r="G196" s="2" t="inlineStr">
         <is>
-          <t>Closest text found (not necessarily enough for 'met'): “Cookies and tracking technologies to improve website functionality and gather analytics. This may include IP addresses, browser types, and usage data. Improve our website’s functionality and performance through analytics tools such as Google Analytics, Google Search Console, and Cloudflare.”</t>
+          <t>[removed: notice text is kept for research only]</t>
         </is>
       </c>
       <c r="H196" s="2" t="inlineStr">
@@ -9856,7 +9856,7 @@
       </c>
       <c r="G197" s="2" t="inlineStr">
         <is>
-          <t>no matching text found</t>
+          <t>[removed: notice text is kept for research only]</t>
         </is>
       </c>
       <c r="H197" s="2" t="inlineStr"/>
@@ -9900,7 +9900,7 @@
       </c>
       <c r="G198" s="2" t="inlineStr">
         <is>
-          <t>“We may use or exchange your information for the following purposes: To authenticate and provide you access to our software and Services and other facilities. To use in our billing systems. To notify you of change of Services, maintenance notifications, school notices and other information. To our third party vendors and our hosting partners in order to provide the necessary Service and related technology required to run the Service. To improve our Service and to track and diagnose problems. To contact you for your reviews and experience using the Service.”</t>
+          <t>[removed: notice text is kept for research only]</t>
         </is>
       </c>
       <c r="H198" s="2" t="inlineStr">
@@ -9948,7 +9948,7 @@
       </c>
       <c r="G199" s="2" t="inlineStr">
         <is>
-          <t>no matching text found</t>
+          <t>[removed: notice text is kept for research only]</t>
         </is>
       </c>
       <c r="H199" s="2" t="inlineStr"/>
@@ -9992,7 +9992,7 @@
       </c>
       <c r="G200" s="2" t="inlineStr">
         <is>
-          <t>no matching text found</t>
+          <t>[removed: notice text is kept for research only]</t>
         </is>
       </c>
       <c r="H200" s="2" t="inlineStr"/>
@@ -10036,7 +10036,7 @@
       </c>
       <c r="G201" s="2" t="inlineStr">
         <is>
-          <t>no matching text found</t>
+          <t>[removed: notice text is kept for research only]</t>
         </is>
       </c>
       <c r="H201" s="2" t="inlineStr"/>
@@ -10080,7 +10080,7 @@
       </c>
       <c r="G202" s="2" t="inlineStr">
         <is>
-          <t>(whole notice) The notice text is in English.</t>
+          <t>[removed: notice text is kept for research only]</t>
         </is>
       </c>
       <c r="H202" s="2" t="inlineStr">
@@ -10128,7 +10128,7 @@
       </c>
       <c r="G203" s="2" t="inlineStr">
         <is>
-          <t>no matching text found</t>
+          <t>[removed: notice text is kept for research only]</t>
         </is>
       </c>
       <c r="H203" s="2" t="inlineStr"/>
@@ -10172,7 +10172,7 @@
       </c>
       <c r="G204" s="2" t="inlineStr">
         <is>
-          <t>no matching text found</t>
+          <t>[removed: notice text is kept for research only]</t>
         </is>
       </c>
       <c r="H204" s="2" t="inlineStr"/>
@@ -10216,7 +10216,7 @@
       </c>
       <c r="G205" s="2" t="inlineStr">
         <is>
-          <t>no matching text found</t>
+          <t>[removed: notice text is kept for research only]</t>
         </is>
       </c>
       <c r="H205" s="2" t="inlineStr"/>
@@ -10260,7 +10260,7 @@
       </c>
       <c r="G206" s="2" t="inlineStr">
         <is>
-          <t>“We are committed to protect the privacy of our students and parents, and ensure that your information remains private and confidential. We will never use, sell, rent, exchange or share your information with any third parties.”</t>
+          <t>[removed: notice text is kept for research only]</t>
         </is>
       </c>
       <c r="H206" s="2" t="inlineStr">
@@ -10308,7 +10308,7 @@
       </c>
       <c r="G207" s="2" t="inlineStr">
         <is>
-          <t>Closest text found (not necessarily enough for 'met'): “We are committed to protect the privacy of our students and parents, and ensure that your information remains private and confidential. We will never use, sell, rent, exchange or share your information with any third parties.”</t>
+          <t>[removed: notice text is kept for research only]</t>
         </is>
       </c>
       <c r="H207" s="2" t="inlineStr">
@@ -10356,7 +10356,7 @@
       </c>
       <c r="G208" s="2" t="inlineStr">
         <is>
-          <t>no matching text found</t>
+          <t>[removed: notice text is kept for research only]</t>
         </is>
       </c>
       <c r="H208" s="2" t="inlineStr"/>
@@ -10400,7 +10400,7 @@
       </c>
       <c r="G209" s="2" t="inlineStr">
         <is>
-          <t>no matching text found</t>
+          <t>[removed: notice text is kept for research only]</t>
         </is>
       </c>
       <c r="H209" s="2" t="inlineStr"/>
@@ -10444,7 +10444,7 @@
       </c>
       <c r="G210" s="2" t="inlineStr">
         <is>
-          <t>no matching text found</t>
+          <t>[removed: notice text is kept for research only]</t>
         </is>
       </c>
       <c r="H210" s="2" t="inlineStr"/>
@@ -10488,7 +10488,7 @@
       </c>
       <c r="G211" s="2" t="inlineStr">
         <is>
-          <t>Closest text found (not necessarily enough for 'met'): “To improve our Service and to track and diagnose problems.”</t>
+          <t>[removed: notice text is kept for research only]</t>
         </is>
       </c>
       <c r="H211" s="2" t="inlineStr">
@@ -10536,7 +10536,7 @@
       </c>
       <c r="G212" s="2" t="inlineStr">
         <is>
-          <t>“The School may collect the information mentioned below directly during the admission process which includes personal and sensitive information. Student’s name, Parents or Guardians name. Email address, telephone or mobile number, postal address, etc. Students age, date of birth, details of family members, siblings, etc. Contact information of relatives, friends, etc., who come into contact with the school. Payment information, if payment information is made through cheque, net banking, credit or debit card, etc. Medical ailment. Future communication preference.”</t>
+          <t>[removed: notice text is kept for research only]</t>
         </is>
       </c>
       <c r="H212" s="2" t="inlineStr">
@@ -10584,7 +10584,7 @@
       </c>
       <c r="G213" s="2" t="inlineStr">
         <is>
-          <t>“We use the collected information for the following purposes: To provide educational services and maintain academic records. To communicate with students, parents, and staff. To ensure the safety and security of our school community. To improve our website and online services.”</t>
+          <t>[removed: notice text is kept for research only]</t>
         </is>
       </c>
       <c r="H213" s="2" t="inlineStr">
@@ -10632,7 +10632,7 @@
       </c>
       <c r="G214" s="2" t="inlineStr">
         <is>
-          <t>no matching text found</t>
+          <t>[removed: notice text is kept for research only]</t>
         </is>
       </c>
       <c r="H214" s="2" t="inlineStr"/>
@@ -10676,7 +10676,7 @@
       </c>
       <c r="G215" s="2" t="inlineStr">
         <is>
-          <t>“We do not store any of your personal information in cookies, web and beacons or other technologies on our computer. Hence, you are not required to provide any personal information through this website unless you choose to do so. We cannot guarantee confidentiality of e-mails and we therefore recommend that you do not send confidential information via e-mail. If for any reason you are concerned that the personal information available at the [NAME], [NAME] is not correct or needs to be changed, you may please contact us for the same.”</t>
+          <t>[removed: notice text is kept for research only]</t>
         </is>
       </c>
       <c r="H215" s="2" t="inlineStr">
@@ -10724,7 +10724,7 @@
       </c>
       <c r="G216" s="2" t="inlineStr">
         <is>
-          <t>no matching text found</t>
+          <t>[removed: notice text is kept for research only]</t>
         </is>
       </c>
       <c r="H216" s="2" t="inlineStr"/>
@@ -10768,7 +10768,7 @@
       </c>
       <c r="G217" s="2" t="inlineStr">
         <is>
-          <t>(whole notice) The notice text is in English.</t>
+          <t>[removed: notice text is kept for research only]</t>
         </is>
       </c>
       <c r="H217" s="2" t="inlineStr">
@@ -10816,7 +10816,7 @@
       </c>
       <c r="G218" s="2" t="inlineStr">
         <is>
-          <t>“[EMAIL] We do not store any of your personal information in cookies, web and beacons or other technologies on our computer. Hence, you are not required to provide any personal information through this website unless you choose to do so. We cannot guarantee confidentiality of e-mails and we therefore recommend that you do not send confidential information via e-mail. If for any reason you are concerned that the personal information available at the [NAME], [NAME] is not correct or needs to be changed, you may please contact us for the same.”</t>
+          <t>[removed: notice text is kept for research only]</t>
         </is>
       </c>
       <c r="H218" s="2" t="inlineStr">
@@ -10864,7 +10864,7 @@
       </c>
       <c r="G219" s="2" t="inlineStr">
         <is>
-          <t>no matching text found</t>
+          <t>[removed: notice text is kept for research only]</t>
         </is>
       </c>
       <c r="H219" s="2" t="inlineStr"/>
@@ -10908,7 +10908,7 @@
       </c>
       <c r="G220" s="2" t="inlineStr">
         <is>
-          <t>no matching text found</t>
+          <t>[removed: notice text is kept for research only]</t>
         </is>
       </c>
       <c r="H220" s="2" t="inlineStr"/>
@@ -10952,7 +10952,7 @@
       </c>
       <c r="G221" s="2" t="inlineStr">
         <is>
-          <t>“Thank you for visiting the [NAME], [NAME]’s website. The School is committed to maintaining your trust by protecting personal information we collect about you, and this statement outlines the school’s policy on how the school uses and manages personal data provided to or collected by the school.”</t>
+          <t>[removed: notice text is kept for research only]</t>
         </is>
       </c>
       <c r="H221" s="2" t="inlineStr">
@@ -11000,7 +11000,7 @@
       </c>
       <c r="G222" s="2" t="inlineStr">
         <is>
-          <t>Closest text found (not necessarily enough for 'met'): “The School may collect information about you from a variety of sources, including information we collect from you directly during pre-admissions, when you intend to admit your child in the [NAME] or otherwise provided directly to us. Generally, we collect information about an individual by way of application form filled out by you, discussion, meetings, interviews and telephone calls during and after the course of a student’s admission at the school.”</t>
+          <t>[removed: notice text is kept for research only]</t>
         </is>
       </c>
       <c r="H222" s="2" t="inlineStr">
@@ -11017,7 +11017,7 @@
       <c r="K222" s="5" t="n"/>
       <c r="L222" s="5" t="inlineStr">
         <is>
-          <t>Line 96 refers to admitting 'your child' and lines 99-104/108 describe collecting and using student data (age, date of birth, medical ailment), so the notice does mention students as children; unsure whether describing collection/use counts as 'how it treats' children's data (Y) or not (N).</t>
+          <t>Line 96 refers to admitting [quote removed] and lines 99-104/108 describe collecting and using student data (age, date of birth, medical ailment), so the notice does mention students as children; unsure whether describing collection/use counts as [quote removed] children's data (Y) or not (N).</t>
         </is>
       </c>
     </row>
@@ -11052,7 +11052,7 @@
       </c>
       <c r="G223" s="2" t="inlineStr">
         <is>
-          <t>no matching text found</t>
+          <t>[removed: notice text is kept for research only]</t>
         </is>
       </c>
       <c r="H223" s="2" t="inlineStr"/>
@@ -11096,7 +11096,7 @@
       </c>
       <c r="G224" s="2" t="inlineStr">
         <is>
-          <t>no matching text found</t>
+          <t>[removed: notice text is kept for research only]</t>
         </is>
       </c>
       <c r="H224" s="2" t="inlineStr"/>
@@ -11140,7 +11140,7 @@
       </c>
       <c r="G225" s="2" t="inlineStr">
         <is>
-          <t>no matching text found</t>
+          <t>[removed: notice text is kept for research only]</t>
         </is>
       </c>
       <c r="H225" s="2" t="inlineStr"/>
@@ -11184,7 +11184,7 @@
       </c>
       <c r="G226" s="2" t="inlineStr">
         <is>
-          <t>Closest text found (not necessarily enough for 'met'): “The cookies are unique bits of computer data that many major websites will transfer to your computer the first time that you visit. Cookies are stored on your hard drive and may be later accessed by the website to track prior usage. Cookies may also be used to deliver customized and personalized services and information by tracking which pages a user has already visited. We do not store any of your personal information in cookies, web and beacons or other technologies on our computer. Hence, you are not required to provide any personal information through this website unless you choose to do so. We cannot guarantee confidentiality of e-mails and we therefore recommend that you do not send confidential information via e-mail. If for any reason you are concerned that the personal information available at the [NAME], [NAME] is not correct or needs to be changed, you may please contact us [...]”</t>
+          <t>[removed: notice text is kept for research only]</t>
         </is>
       </c>
       <c r="H226" s="2" t="inlineStr">
@@ -11232,7 +11232,7 @@
       </c>
       <c r="G227" s="2" t="inlineStr">
         <is>
-          <t>“When you visit our Website, as part of a purchase of one of our courses or by registering on our Website, we may collect a variety of information that you agree to voluntarily provide us via the Website, contact forms, or via a chat or phone session (Personal Identifying Information), such as: Contact Information, such as name, email address, display picture, mailing address, phone number, IP address, geographic location, or phone number; Information to enable us to check and verify your identity, e.g. your date of birth, mark-sheets, or official identification documents, such as Passport/ Aadhaar data/ Voter ID details; Other details such as gender, age to provide you relevant details about financial aid and scholarships; Other details you submit to help us administer the course better; Billing Information, such as debit card number, credit card number and billing address; Unique [...]”</t>
+          <t>[removed: notice text is kept for research only]</t>
         </is>
       </c>
       <c r="H227" s="2" t="inlineStr">
@@ -11280,7 +11280,7 @@
       </c>
       <c r="G228" s="2" t="inlineStr">
         <is>
-          <t>“We will use your personal information to provide, analyse, administer and improve our Services, to provide you with a personalized experience on our Website (especially, by offering you Services that is best suited for you), to contact you about your account and our Services, to provide you customer service, to provide you with personalized marketing and to detect, prevent, mitigate and investigate fraudulent or illegal activities. We further use your personal information to determine your general geographic location, provide localized courses and classes; enhance your user experience; provide you with customized and personalized study material, recommendations; determine your internet service provider; quickly and efficiently respond to your inquiries and requests; to enforce our terms (such as determining free trial eligibility) and to communicate with you concerning our Services (for [...]”</t>
+          <t>[removed: notice text is kept for research only]</t>
         </is>
       </c>
       <c r="H228" s="2" t="inlineStr">
@@ -11328,7 +11328,7 @@
       </c>
       <c r="G229" s="2" t="inlineStr">
         <is>
-          <t>“If you do not wish to receive marketing communications from us, you can write in to us at [EMAIL]”</t>
+          <t>[removed: notice text is kept for research only]</t>
         </is>
       </c>
       <c r="H229" s="2" t="inlineStr">
@@ -11376,7 +11376,7 @@
       </c>
       <c r="G230" s="2" t="inlineStr">
         <is>
-          <t>“This Privacy Policy along with Terms of Use, describes our practices regarding, including your choices in relation to how we collect, store, use, share and secure your personal information across our Website. It also describes your choices regarding use, access and correction of your personal information and your rights in relation to your personal information and how to contact us or supervisory authorities in the event you have a complaint. We may need to retain information even after you have requested us to erase your personal data, terminated your account with us, or have stopped using the Services to ensure compliance with applicable laws or other legal obligations, or to exercise our legal rights. We may also keep your contact information and other details for fraud prevention, for the exercise/defence of a legal claim, or for business compliances such as maintaining accurate [...]”</t>
+          <t>[removed: notice text is kept for research only]</t>
         </is>
       </c>
       <c r="H230" s="2" t="inlineStr">
@@ -11424,7 +11424,7 @@
       </c>
       <c r="G231" s="2" t="inlineStr">
         <is>
-          <t>Closest text found (not necessarily enough for 'met'): “This Privacy Policy along with Terms of Use, describes our practices regarding, including your choices in relation to how we collect, store, use, share and secure your personal information across our Website. It also describes your choices regarding use, access and correction of your personal information and your rights in relation to your personal information and how to contact us or supervisory authorities in the event you have a complaint.”</t>
+          <t>[removed: notice text is kept for research only]</t>
         </is>
       </c>
       <c r="H231" s="2" t="inlineStr">
@@ -11445,7 +11445,7 @@
       </c>
       <c r="L231" s="5" t="inlineStr">
         <is>
-          <t>Line 18: policy says how to contact 'supervisory authorities in the event you have a complaint' (generic authority); lines 117-118 arbitration/courts. Generic route = P.</t>
+          <t>Line 18: policy says how to contact [quote removed] (generic authority); lines 117-118 arbitration/courts. Generic route = P.</t>
         </is>
       </c>
     </row>
@@ -11480,7 +11480,7 @@
       </c>
       <c r="G232" s="2" t="inlineStr">
         <is>
-          <t>(whole notice) The notice text is in English.</t>
+          <t>[removed: notice text is kept for research only]</t>
         </is>
       </c>
       <c r="H232" s="2" t="inlineStr">
@@ -11528,7 +11528,7 @@
       </c>
       <c r="G233" s="2" t="inlineStr">
         <is>
-          <t>“GRIEVANCE OFFICER In accordance with Information Technology Act 2000 and rules made there under, the name and contact details of the Grievance Officer are provided belows: Name: [NAME] Designation: Grievance Officer Email: [EMAIL]”</t>
+          <t>[removed: notice text is kept for research only]</t>
         </is>
       </c>
       <c r="H233" s="2" t="inlineStr">
@@ -11576,7 +11576,7 @@
       </c>
       <c r="G234" s="2" t="inlineStr">
         <is>
-          <t>“GRIEVANCE OFFICER In accordance with Information Technology Act 2000 and rules made there under, the name and contact details of the Grievance Officer are provided belows: Name: [NAME] Designation: Grievance Officer Email: [EMAIL]”</t>
+          <t>[removed: notice text is kept for research only]</t>
         </is>
       </c>
       <c r="H234" s="2" t="inlineStr">
@@ -11624,7 +11624,7 @@
       </c>
       <c r="G235" s="2" t="inlineStr">
         <is>
-          <t>no matching text found</t>
+          <t>[removed: notice text is kept for research only]</t>
         </is>
       </c>
       <c r="H235" s="2" t="inlineStr"/>
@@ -11668,7 +11668,7 @@
       </c>
       <c r="G236" s="2" t="inlineStr">
         <is>
-          <t>“This Privacy Policy discloses the privacy practices for [NAME] (“[NAME]”) with regard to your (a) use of our website, our applications or any products or services in connection with the application, website/products (“Services”) or (b) any modes of registrations or usage of products, including through SD cards, tablets or other storage/transmitting device, including at our physical centers, workshops, events hosted by [NAME]. This Privacy Policy along with Terms of Use, describes our practices regarding, including your choices in relation to how we collect, store, use, share and secure your personal information across our Website. It also describes your choices regarding use, access and correction of your personal information and your rights in relation to your personal information and how to contact us or supervisory authorities in the event you have a complaint.”</t>
+          <t>[removed: notice text is kept for research only]</t>
         </is>
       </c>
       <c r="H236" s="2" t="inlineStr">
@@ -11716,7 +11716,7 @@
       </c>
       <c r="G237" s="2" t="inlineStr">
         <is>
-          <t>“As stated in out in the Terms of Use, you must meet the age requirements for registering and using our Services. Persons who are minors (i.e. a child who has not completed the age of 18 (eighteen) years), un-discharged insolvents etc. are not eligible to register for the Services. As a minor if you wish to use our Services, such use shall be made available to you by your legal guardian or parents, who has agreed to the Terms of Use and this Privacy Policy. In the event a minor utilizes the Services, it is assumed that he/she has obtained the consent of the legal guardian, or parents and such use is made available by the legal guardian or parents. We will not be responsible for any consequence that arises as a result of misuse of any kind that may occur by virtue of any person including a minor registering for the Services provided.”</t>
+          <t>[removed: notice text is kept for research only]</t>
         </is>
       </c>
       <c r="H237" s="2" t="inlineStr">
@@ -11764,7 +11764,7 @@
       </c>
       <c r="G238" s="2" t="inlineStr">
         <is>
-          <t>“As stated in out in the Terms of Use, you must meet the age requirements for registering and using our Services. Persons who are minors (i.e. a child who has not completed the age of 18 (eighteen) years), un-discharged insolvents etc. are not eligible to register for the Services. As a minor if you wish to use our Services, such use shall be made available to you by your legal guardian or parents, who has agreed to the Terms of Use and this Privacy Policy. In the event a minor utilizes the Services, it is assumed that he/she has obtained the consent of the legal guardian, or parents and such use is made available by the legal guardian or parents. We will not be responsible for any consequence that arises as a result of misuse of any kind that may occur by virtue of any person including a minor registering for the Services provided.”</t>
+          <t>[removed: notice text is kept for research only]</t>
         </is>
       </c>
       <c r="H238" s="2" t="inlineStr">
@@ -11812,7 +11812,7 @@
       </c>
       <c r="G239" s="2" t="inlineStr">
         <is>
-          <t>“As stated in out in the Terms of Use, you must meet the age requirements for registering and using our Services. Persons who are minors (i.e. a child who has not completed the age of 18 (eighteen) years), un-discharged insolvents etc. are not eligible to register for the Services. As a minor if you wish to use our Services, such use shall be made available to you by your legal guardian or parents, who has agreed to the Terms of Use and this Privacy Policy. In the event a minor utilizes the Services, it is assumed that he/she has obtained the consent of the legal guardian, or parents and such use is made available by the legal guardian or parents. We will not be responsible for any consequence that arises as a result of misuse of any kind that may occur by virtue of any person including a minor registering for the Services provided. By using the Services, you warrant that all the data [...]”</t>
+          <t>[removed: notice text is kept for research only]</t>
         </is>
       </c>
       <c r="H239" s="2" t="inlineStr">
@@ -11860,7 +11860,7 @@
       </c>
       <c r="G240" s="2" t="inlineStr">
         <is>
-          <t>no matching text found</t>
+          <t>[removed: notice text is kept for research only]</t>
         </is>
       </c>
       <c r="H240" s="2" t="inlineStr"/>
@@ -11904,7 +11904,7 @@
       </c>
       <c r="G241" s="2" t="inlineStr">
         <is>
-          <t>Closest text found (not necessarily enough for 'met'): “We will use your personal information to provide, analyse, administer and improve our Services, to provide you with a personalized experience on our Website (especially, by offering you Services that is best suited for you), to contact you about your account and our Services, to provide you customer service, to provide you with personalized marketing and to detect, prevent, mitigate and investigate fraudulent or illegal activities. It is open for you to customize our usage of your Personal Data to communicate with you, to send you marketing information, how we provide you with customized and relevant advertising, and whether you want to stay signed into your account.”</t>
+          <t>[removed: notice text is kept for research only]</t>
         </is>
       </c>
       <c r="H241" s="2" t="inlineStr">
@@ -11952,7 +11952,7 @@
       </c>
       <c r="G242" s="2" t="inlineStr">
         <is>
-          <t>“Personal Information. By visiting or using the Site, we may collect the following categories of personal information (" personal information ") you provide to us: name; title; email address; postal address; phone number (including your mobile phone number); children's names; job role; marketing responses; admissions follow-ups; and other information you may provide about yourself to the Site or to which you provide us with access via third-party platforms.”</t>
+          <t>[removed: notice text is kept for research only]</t>
         </is>
       </c>
       <c r="H242" s="2" t="inlineStr">
@@ -12000,7 +12000,7 @@
       </c>
       <c r="G243" s="2" t="inlineStr">
         <is>
-          <t>“YOUR INFORMATION We may use your information for the following purposes (" Purposes"), to: provide you with the services, and functionality offered through the Site and fulfil your requests, including, but not limited to; communicate with you about your enquiry or use of the Site, services, or functionality; respond to, or follow up on, your comments and questions, and otherwise provide customer service; communicate with you about special events and other marketing communications; operate and improve the Site, services, and functionality; process and provide events to attend, if applicable; tailor your experience on the Site, including search results and displaying relevant promotions; link or combine with other information we get from third parties to help understand your needs and provide you with better service; perform statistical analysis; protect, investigate, and deter against [...]”</t>
+          <t>[removed: notice text is kept for research only]</t>
         </is>
       </c>
       <c r="H243" s="2" t="inlineStr">
@@ -12048,7 +12048,7 @@
       </c>
       <c r="G244" s="2" t="inlineStr">
         <is>
-          <t>“Your right to withdraw consent. Whenever you have given us your consent to use your personal data, you have the right to change your mind at any time and withdraw that consent.”</t>
+          <t>[removed: notice text is kept for research only]</t>
         </is>
       </c>
       <c r="H244" s="2" t="inlineStr">
@@ -12096,7 +12096,7 @@
       </c>
       <c r="G245" s="2" t="inlineStr">
         <is>
-          <t>“You have the right to request: Access to the personal data we hold about you, free of charge in most cases. The correction of your personal data when incorrect, out of date or incomplete. That we stop using your personal data for direct marketing (either through specific channels, or all channels). That we stop any consent-based processing of your personal data after you withdraw that consent. You can contact us to request to exercise these rights at any time, below.”</t>
+          <t>[removed: notice text is kept for research only]</t>
         </is>
       </c>
       <c r="H245" s="2" t="inlineStr">
@@ -12144,7 +12144,7 @@
       </c>
       <c r="G246" s="2" t="inlineStr">
         <is>
-          <t>“What to do if you're not happy. In the first instance, please talk to us directly so we can resolve any problem or query. You also have the right to contact the Information Commissions Office (ICO) if you have any questions about Data Protection. You can contact them using their help line [PHONE] or at”</t>
+          <t>[removed: notice text is kept for research only]</t>
         </is>
       </c>
       <c r="H246" s="2" t="inlineStr">
@@ -12192,7 +12192,7 @@
       </c>
       <c r="G247" s="2" t="inlineStr">
         <is>
-          <t>(whole notice) The notice text is in English.</t>
+          <t>[removed: notice text is kept for research only]</t>
         </is>
       </c>
       <c r="H247" s="2" t="inlineStr">
@@ -12240,7 +12240,7 @@
       </c>
       <c r="G248" s="2" t="inlineStr">
         <is>
-          <t>“10 CONTACT US If you have any questions about this Policy or information we have collected about you, please Contact Us. We will aim to respond to all queries within 30 days.”</t>
+          <t>[removed: notice text is kept for research only]</t>
         </is>
       </c>
       <c r="H248" s="2" t="inlineStr">
@@ -12288,7 +12288,7 @@
       </c>
       <c r="G249" s="2" t="inlineStr">
         <is>
-          <t>“What to do if you're not happy. In the first instance, please talk to us directly so we can resolve any problem or query. You also have the right to contact the”</t>
+          <t>[removed: notice text is kept for research only]</t>
         </is>
       </c>
       <c r="H249" s="2" t="inlineStr">
@@ -12336,7 +12336,7 @@
       </c>
       <c r="G250" s="2" t="inlineStr">
         <is>
-          <t>“10 CONTACT US If you have any questions about this Policy or information we have collected about you, please Contact Us. We will aim to respond to all queries within 30 days.”</t>
+          <t>[removed: notice text is kept for research only]</t>
         </is>
       </c>
       <c r="H250" s="2" t="inlineStr">
@@ -12384,7 +12384,7 @@
       </c>
       <c r="G251" s="2" t="inlineStr">
         <is>
-          <t>“This privacy policy (this " Policy") explains how personal information is collected, used, and disclosed by [NAME] (collectively, " [NAME], " "[NAME]", " we," " our" or " us"). This Policy applies to visitors and users”</t>
+          <t>[removed: notice text is kept for research only]</t>
         </is>
       </c>
       <c r="H251" s="2" t="inlineStr">
@@ -12432,7 +12432,7 @@
       </c>
       <c r="G252" s="2" t="inlineStr">
         <is>
-          <t>Closest text found (not necessarily enough for 'met'): “information ") you provide to us: name; title; email address; postal address; phone number (including your mobile phone number); children's names; job role; marketing”</t>
+          <t>[removed: notice text is kept for research only]</t>
         </is>
       </c>
       <c r="H252" s="2" t="inlineStr">
@@ -12480,7 +12480,7 @@
       </c>
       <c r="G253" s="2" t="inlineStr">
         <is>
-          <t>no matching text found</t>
+          <t>[removed: notice text is kept for research only]</t>
         </is>
       </c>
       <c r="H253" s="2" t="inlineStr"/>
@@ -12524,7 +12524,7 @@
       </c>
       <c r="G254" s="2" t="inlineStr">
         <is>
-          <t>no matching text found</t>
+          <t>[removed: notice text is kept for research only]</t>
         </is>
       </c>
       <c r="H254" s="2" t="inlineStr"/>
@@ -12568,7 +12568,7 @@
       </c>
       <c r="G255" s="2" t="inlineStr">
         <is>
-          <t>no matching text found</t>
+          <t>[removed: notice text is kept for research only]</t>
         </is>
       </c>
       <c r="H255" s="2" t="inlineStr"/>
@@ -12612,7 +12612,7 @@
       </c>
       <c r="G256" s="2" t="inlineStr">
         <is>
-          <t>Closest text found (not necessarily enough for 'met'): “Combined Information. We may combine your personal information with device information and location information (with your consent, where required) to serve you specifically, such as to deliver a service to you according to your preferences or restrictions, or for advertising or advertising targeting purposes. When we”</t>
+          <t>[removed: notice text is kept for research only]</t>
         </is>
       </c>
       <c r="H256" s="2" t="inlineStr">
@@ -12660,7 +12660,7 @@
       </c>
       <c r="G257" s="2" t="inlineStr">
         <is>
-          <t>“application. In particular, the School may collect the following types of personal information: • name, address, nationality, contact details, including email and contact number and employment/ professional details; • information that one would usually include in a resume, including name, contact details including e-mail address and mobile number, work experience, educational qualifications, data relating to your current and past remuneration or salary, a copy of your resume, etc. in case of a job applicant or an employee; • details of pupils, parents / guardians and other members of pupils’ families, governors, suppliers and other individuals that we communicate with, including name, residential address, email address, contact number, nationality, age, past and present educational records, qualification records, etc., when you apply for admission.”</t>
+          <t>[removed: notice text is kept for research only]</t>
         </is>
       </c>
       <c r="H257" s="2" t="inlineStr">
@@ -12708,7 +12708,7 @@
       </c>
       <c r="G258" s="2" t="inlineStr">
         <is>
-          <t>“which you interact with the School. The School may use or process personal information for the following purposes: • for providing the services requested, including providing job/admission and to contact you in relation to the same and when otherwise necessary; • for enabling school council to fulfil its objectives and functions, including for assessing applicants’ job application / admission application; • for departmental research or school statistics purposes;”</t>
+          <t>[removed: notice text is kept for research only]</t>
         </is>
       </c>
       <c r="H258" s="2" t="inlineStr">
@@ -12756,7 +12756,7 @@
       </c>
       <c r="G259" s="2" t="inlineStr">
         <is>
-          <t>“At any time while availing the services provided by the School, you will have the option to withdraw your consent to the use/disclosure/retention of such SPDI, provided that the same is communicated to the School in writing. In such an event, the School will be entitled to immediately terminate the services offered and/or your access to the website/ mobile applications, as the case maybe.”</t>
+          <t>[removed: notice text is kept for research only]</t>
         </is>
       </c>
       <c r="H259" s="2" t="inlineStr">
@@ -12804,7 +12804,7 @@
       </c>
       <c r="G260" s="2" t="inlineStr">
         <is>
-          <t>“Access and Accuracy: The information provider has a right to review, update and correct their personal information that the School holds. Should the information provider need to update or correct any Personal Information provided by them, please contact us at the following e-mail address [EMAIL] and the School will make reasonable efforts to incorporate the changes in your personal information that we hold as soon as.”</t>
+          <t>[removed: notice text is kept for research only]</t>
         </is>
       </c>
       <c r="H260" s="2" t="inlineStr">
@@ -12852,7 +12852,7 @@
       </c>
       <c r="G261" s="2" t="inlineStr">
         <is>
-          <t>no matching text found</t>
+          <t>[removed: notice text is kept for research only]</t>
         </is>
       </c>
       <c r="H261" s="2" t="inlineStr"/>
@@ -12896,7 +12896,7 @@
       </c>
       <c r="G262" s="2" t="inlineStr">
         <is>
-          <t>(whole notice) The notice text is in English.</t>
+          <t>[removed: notice text is kept for research only]</t>
         </is>
       </c>
       <c r="H262" s="2" t="inlineStr">
@@ -12944,7 +12944,7 @@
       </c>
       <c r="G263" s="2" t="inlineStr">
         <is>
-          <t>“Grievances and Complaints: Any grievances or complaints in relation to the processing of any personal information by the School, may be addressed to the School’s Grievance Officer Mr [NAME] at the following email address: [EMAIL]”</t>
+          <t>[removed: notice text is kept for research only]</t>
         </is>
       </c>
       <c r="H263" s="2" t="inlineStr">
@@ -12992,7 +12992,7 @@
       </c>
       <c r="G264" s="2" t="inlineStr">
         <is>
-          <t>“Grievances and Complaints: Any grievances or complaints in relation to the processing of any personal information by the School, may be addressed to the School’s Grievance Officer Mr [NAME] at the following email address: [EMAIL]”</t>
+          <t>[removed: notice text is kept for research only]</t>
         </is>
       </c>
       <c r="H264" s="2" t="inlineStr">
@@ -13040,7 +13040,7 @@
       </c>
       <c r="G265" s="2" t="inlineStr">
         <is>
-          <t>no matching text found</t>
+          <t>[removed: notice text is kept for research only]</t>
         </is>
       </c>
       <c r="H265" s="2" t="inlineStr"/>
@@ -13084,7 +13084,7 @@
       </c>
       <c r="G266" s="2" t="inlineStr">
         <is>
-          <t>“[NAME], under the aegis of ‘[NAME]’ (“the School”), aims to ensure that all personal data and information collected in relation to the School operations, is stored, processed and deleted in accordance with the laws and regulations applicable to the School. The School believes that the protection of personal data is critical to maintain a secure environment.”</t>
+          <t>[removed: notice text is kept for research only]</t>
         </is>
       </c>
       <c r="H266" s="2" t="inlineStr">
@@ -13132,7 +13132,7 @@
       </c>
       <c r="G267" s="2" t="inlineStr">
         <is>
-          <t>Closest text found (not necessarily enough for 'met'): “• details of pupils, parents / guardians and other members of pupils’ families, governors, suppliers and other individuals that we communicate with, including name, residential address, email address, contact number, nationality, age, past and present educational records, qualification records, etc., when you apply for admission.”</t>
+          <t>[removed: notice text is kept for research only]</t>
         </is>
       </c>
       <c r="H267" s="2" t="inlineStr">
@@ -13180,7 +13180,7 @@
       </c>
       <c r="G268" s="2" t="inlineStr">
         <is>
-          <t>no matching text found</t>
+          <t>[removed: notice text is kept for research only]</t>
         </is>
       </c>
       <c r="H268" s="2" t="inlineStr"/>
@@ -13224,7 +13224,7 @@
       </c>
       <c r="G269" s="2" t="inlineStr">
         <is>
-          <t>no matching text found</t>
+          <t>[removed: notice text is kept for research only]</t>
         </is>
       </c>
       <c r="H269" s="2" t="inlineStr"/>
@@ -13268,7 +13268,7 @@
       </c>
       <c r="G270" s="2" t="inlineStr">
         <is>
-          <t>no matching text found</t>
+          <t>[removed: notice text is kept for research only]</t>
         </is>
       </c>
       <c r="H270" s="2" t="inlineStr"/>
@@ -13312,7 +13312,7 @@
       </c>
       <c r="G271" s="2" t="inlineStr">
         <is>
-          <t>no matching text found</t>
+          <t>[removed: notice text is kept for research only]</t>
         </is>
       </c>
       <c r="H271" s="2" t="inlineStr"/>
@@ -13356,7 +13356,7 @@
       </c>
       <c r="G272" s="2" t="inlineStr">
         <is>
-          <t>“While using Our Service, We may ask You to provide Us with certain personally identifiable information that can be used to contact or identify You. Personally identifiable information may include, but is not limited to: Email address First name and last name Phone number Address, State, Province, ZIP/Postal code, City Usage Data Usage Data Usage Data may include information such as Your Device's Internet Protocol address (e.g. IP address), browser type, browser version, the pages of our Service that You visit, the time and date of Your visit, the time spent on those pages, unique device identifiers and other diagnostic data.”</t>
+          <t>[removed: notice text is kept for research only]</t>
         </is>
       </c>
       <c r="H272" s="2" t="inlineStr">
@@ -13404,7 +13404,7 @@
       </c>
       <c r="G273" s="2" t="inlineStr">
         <is>
-          <t>“The Company may use Personal Data for the following purposes: To provide and maintain our Service , including to monitor the usage of our Service. To manage Your Account: to manage Your registration as a user of the Service. The Personal Data You provide can give You access to different functionalities of the Service that are available to You as a registered user. For the performance of a contract: the development, compliance and undertaking of the purchase contract for the products, items or services You have purchased or of any other contract with Us through the Service. To contact You: To contact You by email, telephone calls, SMS, or other equivalent forms of electronic communication, such as a mobile application's push notifications regarding updates or informative communications related to the functionalities, products or contracted services, including the security updates, when [...]”</t>
+          <t>[removed: notice text is kept for research only]</t>
         </is>
       </c>
       <c r="H273" s="2" t="inlineStr">
@@ -13452,7 +13452,7 @@
       </c>
       <c r="G274" s="2" t="inlineStr">
         <is>
-          <t>Closest text found (not necessarily enough for 'met'): “You can enable or disable access to this information at any time, through Your Device settings.”</t>
+          <t>[removed: notice text is kept for research only]</t>
         </is>
       </c>
       <c r="H274" s="2" t="inlineStr">
@@ -13508,7 +13508,7 @@
       </c>
       <c r="G275" s="2" t="inlineStr">
         <is>
-          <t>“Delete Your Personal Data You have the right to delete or request that We assist in deleting the Personal Data that We have collected about You. Our Service may give You the ability to delete certain information about You from within the Service. You may update, amend, or delete Your information at any time by signing in to Your Account, if you have one, and visiting the account settings section that allows you to manage Your personal information. You may also contact Us to request access to, correct, or delete any personal information that You have provided to Us.”</t>
+          <t>[removed: notice text is kept for research only]</t>
         </is>
       </c>
       <c r="H275" s="2" t="inlineStr">
@@ -13556,7 +13556,7 @@
       </c>
       <c r="G276" s="2" t="inlineStr">
         <is>
-          <t>no matching text found</t>
+          <t>[removed: notice text is kept for research only]</t>
         </is>
       </c>
       <c r="H276" s="2" t="inlineStr"/>
@@ -13600,7 +13600,7 @@
       </c>
       <c r="G277" s="2" t="inlineStr">
         <is>
-          <t>(whole notice) The notice text is in English.</t>
+          <t>[removed: notice text is kept for research only]</t>
         </is>
       </c>
       <c r="H277" s="2" t="inlineStr">
@@ -13648,7 +13648,7 @@
       </c>
       <c r="G278" s="2" t="inlineStr">
         <is>
-          <t>“If you have any questions about this Privacy Policy, You can contact us: By phone number: [PHONE]”</t>
+          <t>[removed: notice text is kept for research only]</t>
         </is>
       </c>
       <c r="H278" s="2" t="inlineStr">
@@ -13696,7 +13696,7 @@
       </c>
       <c r="G279" s="2" t="inlineStr">
         <is>
-          <t>no matching text found</t>
+          <t>[removed: notice text is kept for research only]</t>
         </is>
       </c>
       <c r="H279" s="2" t="inlineStr"/>
@@ -13740,7 +13740,7 @@
       </c>
       <c r="G280" s="2" t="inlineStr">
         <is>
-          <t>no matching text found</t>
+          <t>[removed: notice text is kept for research only]</t>
         </is>
       </c>
       <c r="H280" s="2" t="inlineStr"/>
@@ -13784,7 +13784,7 @@
       </c>
       <c r="G281" s="2" t="inlineStr">
         <is>
-          <t>“This Privacy Policy describes Our policies and procedures on the collection, use and disclosure of Your information when You use the Service and tells You about Your privacy rights and how the law protects You.”</t>
+          <t>[removed: notice text is kept for research only]</t>
         </is>
       </c>
       <c r="H281" s="2" t="inlineStr">
@@ -13832,7 +13832,7 @@
       </c>
       <c r="G282" s="2" t="inlineStr">
         <is>
-          <t>“Children's Privacy Our Service does not address anyone under the age of 13. We do not knowingly collect personally identifiable information from anyone under the age of 13. If You are a parent or guardian and You are aware that Your child has provided Us with Personal Data, please contact Us. If We become aware that We have collected Personal Data from anyone under the age of 13 without verification of parental consent, We take steps to remove that information from Our servers.”</t>
+          <t>[removed: notice text is kept for research only]</t>
         </is>
       </c>
       <c r="H282" s="2" t="inlineStr">
@@ -13880,7 +13880,7 @@
       </c>
       <c r="G283" s="2" t="inlineStr">
         <is>
-          <t>“Our Service does not address anyone under the age of 13. We do not knowingly collect personally identifiable information from anyone under the age of 13. If You are a parent or guardian and You are aware that Your child has provided Us with Personal Data, please contact Us. If We become aware that We have collected Personal Data from anyone under the age of 13 without verification of parental consent, We take steps to remove that information from Our servers.”</t>
+          <t>[removed: notice text is kept for research only]</t>
         </is>
       </c>
       <c r="H283" s="2" t="inlineStr">
@@ -13928,7 +13928,7 @@
       </c>
       <c r="G284" s="2" t="inlineStr">
         <is>
-          <t>“Our Service does not address anyone under the age of 13. We do not knowingly collect personally identifiable information from anyone under the age of 13. If You are a parent or guardian and You are aware that Your child has provided Us with Personal Data, please contact Us. If We become aware that We have collected Personal Data from anyone under the age of 13 without verification of parental consent, We take steps to remove that information from Our servers. If We need to rely on consent as a legal basis for processing Your information and Your country requires consent from a parent, We may require Your parent's consent before We collect and use that information.”</t>
+          <t>[removed: notice text is kept for research only]</t>
         </is>
       </c>
       <c r="H284" s="2" t="inlineStr">
@@ -13976,7 +13976,7 @@
       </c>
       <c r="G285" s="2" t="inlineStr">
         <is>
-          <t>Closest text found (not necessarily enough for 'met'): “Our Service does not address anyone under the age of 13. We do not knowingly collect personally identifiable information from anyone under the age of 13. If You are a parent or guardian and You are aware that Your child has provided Us with Personal Data, please contact Us. If We become aware that We have collected Personal Data from anyone under the age of 13 without verification of parental consent, We take steps to remove that information from Our servers.”</t>
+          <t>[removed: notice text is kept for research only]</t>
         </is>
       </c>
       <c r="H285" s="2" t="inlineStr">
@@ -13997,7 +13997,7 @@
       </c>
       <c r="L285" s="5" t="inlineStr">
         <is>
-          <t>Line 122: data removed if collected 'without verification of parental consent' = says it verifies, no method (P); CB-033 K4 was coded P on the same clause.</t>
+          <t>Line 122: data removed if collected [quote removed] = says it verifies, no method (P); CB-033 K4 was coded P on the same clause.</t>
         </is>
       </c>
     </row>
@@ -14032,7 +14032,7 @@
       </c>
       <c r="G286" s="2" t="inlineStr">
         <is>
-          <t>no matching text found</t>
+          <t>[removed: notice text is kept for research only]</t>
         </is>
       </c>
       <c r="H286" s="2" t="inlineStr"/>

</xml_diff>

<commit_message>
Apply the final check of the 19 school notices: all 285 codes checked (met-or-not 279/285, kappa 0.951; 18 differences, all where the first pass was stricter), final codes and change log rebuilt from the sheet by checks/apply_check.py, public sheet without notice quotes, re-run tables, figures and results summary
</commit_message>
<xml_diff>
--- a/checks/11-check-sheet.filled.xlsx
+++ b/checks/11-check-sheet.filled.xlsx
@@ -1515,11 +1515,19 @@
       <c r="I19" s="2" t="inlineStr"/>
       <c r="J19" s="5" t="inlineStr">
         <is>
-          <t>Y</t>
-        </is>
-      </c>
-      <c r="K19" s="5" t="n"/>
-      <c r="L19" s="5" t="n"/>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="K19" s="5" t="inlineStr">
+        <is>
+          <t>P</t>
+        </is>
+      </c>
+      <c r="L19" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Consent is by use of the site (10). No statement that consent can be withdrawn, so not Y. The ad-cookie decline via a third-party link (31) and browser cookie settings (43) alone would be N, consistent with CB-033 (analytics opt-out add-on, N) and GV-007 (device settings, N). But line 56 states a right to object to processing, with an e-mail channel for exercising rights (58). Objecting to processing is an opt-out of processing, which the P limb covers ('states a right to withdraw/opt out'). It </t>
+        </is>
+      </c>
     </row>
     <row r="20">
       <c r="A20" s="2" t="n">
@@ -2299,13 +2307,17 @@
       <c r="I35" s="2" t="inlineStr"/>
       <c r="J35" s="5" t="inlineStr">
         <is>
-          <t>?</t>
-        </is>
-      </c>
-      <c r="K35" s="5" t="n"/>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="K35" s="5" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
       <c r="L35" s="5" t="inlineStr">
         <is>
-          <t>Rights to access, correct and delete are named (lines 106-108); the only means are account login for contact details (lines 105-106) and the general [quote removed] (lines 129-132). Unsure whether that is a means to request the rights (Y) or rights with no means (P).</t>
+          <t>Access, correction and deletion are named (106-108). A portal means is given: [quote removed] to keep information accurate and up to date (105-106). Lines 129-132 give contact for questions about data processing. The rule's list of means includes 'portal', and the same structure (account sign-in plus contact) is coded Y at GV-007 (row 274). So both limbs of Y are met. A's point (the login covers contact info only) is about scope, but the rule does not ask for a means for every ri</t>
         </is>
       </c>
     </row>
@@ -5119,13 +5131,17 @@
       <c r="I95" s="2" t="inlineStr"/>
       <c r="J95" s="5" t="inlineStr">
         <is>
-          <t>?</t>
-        </is>
-      </c>
-      <c r="K95" s="5" t="n"/>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="K95" s="5" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
       <c r="L95" s="5" t="inlineStr">
         <is>
-          <t>Line 30 names export and erasure with no channel (P), but line 27 says registered users can see, edit or delete their data in their profile at any time, which may count as a portal means (Y).</t>
+          <t>Under the heading [quote removed] (28), the notice names the right to receive an export of one's data (access) and to request erasure (30). Line 27 gives a self-service means: registered users [quote removed] in their user profile. That is an in-account portal, which covers access, correction and erasure directly. Rights named plus a portal means meets Y, consistent with GV-007 (row 274) and CB-025 (row 34). The rule can dec</t>
         </is>
       </c>
     </row>
@@ -6507,7 +6523,11 @@
         </is>
       </c>
       <c r="K125" s="5" t="n"/>
-      <c r="L125" s="5" t="n"/>
+      <c r="L125" s="5" t="inlineStr">
+        <is>
+          <t>The only rights-related text is [quote removed] (148), under [quote removed] (143). There is a means (account login), but no right of access, correction or erasure is named as a right. The text describes a single update function for self-entered data. That fits the P limb ('a means ... with no rights named'). It matches how the sheet codes bare [quote removed] clauses without rights language as P (CB-</t>
+        </is>
+      </c>
     </row>
     <row r="126">
       <c r="A126" s="2" t="n">
@@ -7167,11 +7187,19 @@
       <c r="I139" s="2" t="inlineStr"/>
       <c r="J139" s="5" t="inlineStr">
         <is>
-          <t>Y</t>
-        </is>
-      </c>
-      <c r="K139" s="5" t="n"/>
-      <c r="L139" s="5" t="n"/>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="K139" s="5" t="inlineStr">
+        <is>
+          <t>P</t>
+        </is>
+      </c>
+      <c r="L139" s="5" t="inlineStr">
+        <is>
+          <t>Processing rests on consent (18: [quote removed]). Line 21 says that when purposes change, [quote removed]. That is a stated opt-out or refusal of consent-based processing, and no channel is given. This is exactly the P limb ('states a right to withdraw/opt out with no channel'). It is narrower than full withdrawal and has no channel, so not Y. It is more than nothing, so not N. Coded the</t>
+        </is>
+      </c>
     </row>
     <row r="140">
       <c r="A140" s="2" t="n">
@@ -11011,13 +11039,17 @@
       <c r="I222" s="2" t="inlineStr"/>
       <c r="J222" s="5" t="inlineStr">
         <is>
-          <t>?</t>
-        </is>
-      </c>
-      <c r="K222" s="5" t="n"/>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="K222" s="5" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
       <c r="L222" s="5" t="inlineStr">
         <is>
-          <t>Line 96 refers to admitting [quote removed] and lines 99-104/108 describe collecting and using student data (age, date of birth, medical ailment), so the notice does mention students as children; unsure whether describing collection/use counts as [quote removed] children's data (Y) or not (N).</t>
+          <t xml:space="preserve">The rule's parenthetical makes the deciding question whether the notice mentions students as children. Line 96 does, addressing parents who [quote removed] and describing collection [quote removed]. The notice then sets out the child/student data collected from parents: student's name, age, date of birth, medical ailment (99-104). It gives the uses: educational services, academic records, communicating with students (106-111). So it states how </t>
         </is>
       </c>
     </row>
@@ -11391,7 +11423,11 @@
         </is>
       </c>
       <c r="K230" s="5" t="n"/>
-      <c r="L230" s="5" t="n"/>
+      <c r="L230" s="5" t="inlineStr">
+        <is>
+          <t>Line 18 says the policy [quote removed], and line 49 mentions requests to erase. So access, correction and erasure are referred to. But the notice never says how to exercise them. The grievance officer e-mail (99-106) and the same address at 64-65, 84-85, 111-112 are offered only for account abuse, marketing opt-out, Terms violations, account termination and IT Act grievances, never for access, correction or erasure requests. Y ne</t>
+        </is>
+      </c>
     </row>
     <row r="231">
       <c r="A231" s="2" t="n">

</xml_diff>